<commit_message>
QS_DAM: dai trong 1 nhanh kieu DCE, so hieu thep C theo be rong thuc dung
- Dai trong mac dinh kieu DCE: dai 1 nhanh tai moi thanh giua lop 1 tren (moc tren 135 do / 6d
  vong qua thanh tren, chan duoi 90 do / 12d), ve o MC ngang + 1 tag chung, thong ke va shop dai.
  QS_DAMSET trang 2: kieu dai trong (1 nhanh / dai kin), goc + L moc tren, L chan duoi.
- So hieu thep C do / dai C noi thep gia chi cap cho be rong dam thuc co dung (het nhay so);
  tag MC ngang lay be rong tai giua thanh nhu thong ke.
- Sua ban kinh bo tron hinh dai 1 nhanh tren shop.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VnufFRFDfSW7EG6WSRTNkK
</commit_message>
<xml_diff>
--- a/QS_DAM_NhapLieu.xlsx
+++ b/QS_DAM_NhapLieu.xlsx
@@ -881,7 +881,8 @@
       <text>
         <t>DÒNG 27
 • GỐI: độ lệch trục so với tim gối (mm).
-• NHỊP: đai trong 6-100/200 (để trống: tự thêm đai trong khi lớp 1 trên ≥ 4 thanh)
+• NHỊP: đai trong 6-100/200 (để trống: tự thêm khi lớp 1 trên ≥ 4 thanh). Kiểu đai trong chọn ở QS_DAMSET trang 2:
+  1 nhánh tại mỗi thanh giữa (như DCE) hoặc đai kín ôm thanh 2 và n-1.
   và/hoặc mối nối bắt buộc: T, B, T/B, TL, TR, BL, BR. Ví dụ 6-100/200/B.</t>
       </text>
     </comment>
@@ -1055,7 +1056,8 @@
       <text>
         <t>DÒNG 27
 • GỐI: độ lệch trục so với tim gối (mm).
-• NHỊP: đai trong 6-100/200 (để trống: tự thêm đai trong khi lớp 1 trên ≥ 4 thanh)
+• NHỊP: đai trong 6-100/200 (để trống: tự thêm khi lớp 1 trên ≥ 4 thanh). Kiểu đai trong chọn ở QS_DAMSET trang 2:
+  1 nhánh tại mỗi thanh giữa (như DCE) hoặc đai kín ôm thanh 2 và n-1.
   và/hoặc mối nối bắt buộc: T, B, T/B, TL, TR, BL, BR. Ví dụ 6-100/200/B.</t>
       </text>
     </comment>
@@ -1595,7 +1597,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="58" customHeight="1">
+    <row r="17" ht="71.5" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>DÒNG 27</t>
@@ -1605,7 +1607,8 @@
         <is>
           <t>DÒNG 27
 • GỐI: độ lệch trục so với tim gối (mm).
-• NHỊP: đai trong 6-100/200 (để trống: tự thêm đai trong khi lớp 1 trên ≥ 4 thanh)
+• NHỊP: đai trong 6-100/200 (để trống: tự thêm khi lớp 1 trên ≥ 4 thanh). Kiểu đai trong chọn ở QS_DAMSET trang 2:
+  1 nhánh tại mỗi thanh giữa (như DCE) hoặc đai kín ôm thanh 2 và n-1.
   và/hoặc mối nối bắt buộc: T, B, T/B, TL, TR, BL, BR. Ví dụ 6-100/200/B.</t>
         </is>
       </c>

</xml_diff>

<commit_message>
QS_DAM: dai trong tai dai gia cuong dam phu, chieu dai dai C bo qua doan uon
- Moi dai gia cuong dam phu (vd 10t10a50) cong them bo dai trong / dai 1 nhanh nhu vi tri dai
  thuong (QS_DAMSET trang 2: DAITRONGGC, mac dinh bat).
- Chieu dai cat dai C va dai 1 nhanh: 'cong doan' = cong kich thuoc ngoai cac doan thang, bo qua
  phan uon (giong DCE: C 60+270+120 = 450, 1 nhanh 72+870+144 = 1085) hoac 'theo tim' (tru uon).
- Tach phan tinh dai trong thanh ham dung chung cho vung dai va dai gia cuong.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VnufFRFDfSW7EG6WSRTNkK
</commit_message>
<xml_diff>
--- a/QS_DAM_NhapLieu.xlsx
+++ b/QS_DAM_NhapLieu.xlsx
@@ -897,7 +897,8 @@
       <text>
         <t>DÒNG 29
 • GỐI: khoảng cách từ TIM gối tới tim dầm giao trong nhịp phải (2000 hoặc 2000/5000).
-• NHỊP: đai gia cường tại dầm giao: 8t8a50 (chia 2 bên), 8t8a50L / 8t8a50R (1 bên), 8u8a50 (chữ u = đai U).</t>
+• NHỊP: đai gia cường tại dầm giao: 8t8a50 (chia 2 bên), 8t8a50L / 8t8a50R (1 bên), 8u8a50 (chữ u = đai U).
+  Mỗi đai gia cường có thêm bộ đai trong / đai 1 nhánh như đai thường (tắt được ở QS_DAMSET trang 2).</t>
       </text>
     </comment>
     <comment ref="A30" authorId="0" shapeId="0">
@@ -1072,7 +1073,8 @@
       <text>
         <t>DÒNG 29
 • GỐI: khoảng cách từ TIM gối tới tim dầm giao trong nhịp phải (2000 hoặc 2000/5000).
-• NHỊP: đai gia cường tại dầm giao: 8t8a50 (chia 2 bên), 8t8a50L / 8t8a50R (1 bên), 8u8a50 (chữ u = đai U).</t>
+• NHỊP: đai gia cường tại dầm giao: 8t8a50 (chia 2 bên), 8t8a50L / 8t8a50R (1 bên), 8u8a50 (chữ u = đai U).
+  Mỗi đai gia cường có thêm bộ đai trong / đai 1 nhánh như đai thường (tắt được ở QS_DAMSET trang 2).</t>
       </text>
     </comment>
     <comment ref="A30" authorId="0" shapeId="0">
@@ -1627,7 +1629,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="44.5" customHeight="1">
+    <row r="19" ht="58" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
           <t>DÒNG 29</t>
@@ -1637,7 +1639,8 @@
         <is>
           <t>DÒNG 29
 • GỐI: khoảng cách từ TIM gối tới tim dầm giao trong nhịp phải (2000 hoặc 2000/5000).
-• NHỊP: đai gia cường tại dầm giao: 8t8a50 (chia 2 bên), 8t8a50L / 8t8a50R (1 bên), 8u8a50 (chữ u = đai U).</t>
+• NHỊP: đai gia cường tại dầm giao: 8t8a50 (chia 2 bên), 8t8a50L / 8t8a50R (1 bên), 8u8a50 (chữ u = đai U).
+  Mỗi đai gia cường có thêm bộ đai trong / đai 1 nhánh như đai thường (tắt được ở QS_DAMSET trang 2).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
QS_DAM: coupler cho keo ra ngoai mep dam, so le 2 doan (vd 100/300)
- Thep cho kieu COUPLER: L cho = 0 (tai mep) | 100 | 100/300 -> ceil(n/2) thanh ra ngoai 100,
  con lai 300 ; AUTO lay QS_DAMSET trang 3 (CPLL, mac dinh 0 = tai mep nhu cu).
- MC doc: ky hieu coupler tai dau thanh (ngoai mep), dim tung doan ra ngoai ; shop cat du chieu dai
  va ve coupler tai dau thanh ; dem coupler theo dau thanh tai / ngoai mep dam.
- Excel: goi y L cho cho coupler (0 / 100 / 100/300), cap nhat huong dan.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VnufFRFDfSW7EG6WSRTNkK
</commit_message>
<xml_diff>
--- a/QS_DAM_NhapLieu.xlsx
+++ b/QS_DAM_NhapLieu.xlsx
@@ -788,7 +788,7 @@
       <text>
         <t>THÉP CHỜ 2 ĐẦU DẦM (khi đầu dầm là mạch ngừng, chờ sang zone / đợt đổ sau)
 • Cho thang: thép kéo thẳng ra ngoài đầu dầm đoạn L chờ, không bẻ ke.
-• Coupler: thép dừng tại mép, vẽ ký hiệu coupler.
+• Coupler: thép dừng tại mép (L chờ = 0) hoặc kéo ra ngoài mép: 100, hoặc so le 100/300 (½ số thanh 100, ½ số thanh 300).
 • So le: 1/2 số thanh chờ L, 1/2 chờ 2L + KC mối nối.
 Bản vẽ có nét khuất dầm zone sau, đường MẠCH NGỪNG, dim L chờ; QS_SHOPDAM cắt đúng chiều dài.
 Để trống = theo QS_DAMSET.</t>
@@ -964,7 +964,7 @@
       <text>
         <t>THÉP CHỜ 2 ĐẦU DẦM (khi đầu dầm là mạch ngừng, chờ sang zone / đợt đổ sau)
 • Cho thang: thép kéo thẳng ra ngoài đầu dầm đoạn L chờ, không bẻ ke.
-• Coupler: thép dừng tại mép, vẽ ký hiệu coupler.
+• Coupler: thép dừng tại mép (L chờ = 0) hoặc kéo ra ngoài mép: 100, hoặc so le 100/300 (½ số thanh 100, ½ số thanh 300).
 • So le: 1/2 số thanh chờ L, 1/2 chờ 2L + KC mối nối.
 Bản vẽ có nét khuất dầm zone sau, đường MẠCH NGỪNG, dim L chờ; QS_SHOPDAM cắt đúng chiều dài.
 Để trống = theo QS_DAMSET.</t>
@@ -1428,7 +1428,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>• THÉP CHỜ 2 ĐẦU DẦM (S3:T7): kiểu (Khong / Cho thang / Coupler), lớp (TBG, TB, T, B), thanh (Tat ca / Chay suot), L chờ (AUTO / 40d / 1200), so le.
+          <t>• THÉP CHỜ 2 ĐẦU DẦM (S3:T7): kiểu (Khong / Cho thang / Coupler), lớp (TBG, TB, T, B), thanh (Tat ca / Chay suot), L chờ (AUTO / 40d / 1200; coupler 0 / 100 / 100/300 so le), so le.
 • TÙY CHỌN SÀN (Y2:Y3): tai sàn 2 ben / Trai / Phai / Khong, sàn lật – dùng khi F7 chỉ là số (nhập mã DCE 150/1, _150 thì bỏ qua Y2:Y3).
 • Dòng 33-35: tọa độ trục, KC trục-trục tính từ bề rộng gối + Ltt + lệch trục; nhập KC trục mặt bằng (dòng 34) → Ltt suy ra (dòng 35, vàng nếu lệch Ltt đang nhập).
 • Dòng 37-42: kiểm tra As (cm²) bố trí / yêu cầu – thép chạy suốt hiệu dụng (có tính đổi thép dòng 23/25) + tăng cường lớp 1..5; gối tách trái/phải.
@@ -13524,8 +13524,8 @@
     <dataValidation sqref="S5 T5" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="QS_DAM" error="Chọn giá trị trong danh sách." promptTitle="Thanh được chờ" prompt="Tat ca = mọi thanh tới đầu dầm&#10;Chay suot = chỉ thép chạy suốt" type="list">
       <formula1>LIST!$U$2:$U$3</formula1>
     </dataValidation>
-    <dataValidation sqref="S6 T6" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="L chờ" prompt="AUTO = L nối ngoài vùng theo bảng QS_DAMNOI · 40d · 1200 (mm)" type="list">
-      <formula1>LIST!$V$2:$V$5</formula1>
+    <dataValidation sqref="S6 T6" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="L chờ" prompt="Chờ thẳng: AUTO = L nối ngoài vùng · 40d · 1200 (mm)&#10;Coupler: đoạn ra ngoài mép 0 · 100 · 100/300 = so le (½ thanh 100, ½ thanh 300); AUTO = QS_DAMSET" type="list">
+      <formula1>LIST!$V$2:$V$8</formula1>
     </dataValidation>
     <dataValidation sqref="S7 T7" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="QS_DAM" error="Chọn giá trị trong danh sách." promptTitle="Chờ so le 50%" prompt="Co = 1/2 số thanh chờ L, 1/2 chờ 2L + KC mối nối" type="list">
       <formula1>LIST!$W$2:$W$3</formula1>
@@ -24770,8 +24770,8 @@
     <dataValidation sqref="S5 T5" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="QS_DAM" error="Chọn giá trị trong danh sách." promptTitle="Thanh được chờ" prompt="Tat ca = mọi thanh tới đầu dầm&#10;Chay suot = chỉ thép chạy suốt" type="list">
       <formula1>LIST!$U$2:$U$3</formula1>
     </dataValidation>
-    <dataValidation sqref="S6 T6" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="L chờ" prompt="AUTO = L nối ngoài vùng theo bảng QS_DAMNOI · 40d · 1200 (mm)" type="list">
-      <formula1>LIST!$V$2:$V$5</formula1>
+    <dataValidation sqref="S6 T6" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="L chờ" prompt="Chờ thẳng: AUTO = L nối ngoài vùng · 40d · 1200 (mm)&#10;Coupler: đoạn ra ngoài mép 0 · 100 · 100/300 = so le (½ thanh 100, ½ thanh 300); AUTO = QS_DAMSET" type="list">
+      <formula1>LIST!$V$2:$V$8</formula1>
     </dataValidation>
     <dataValidation sqref="S7 T7" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="QS_DAM" error="Chọn giá trị trong danh sách." promptTitle="Chờ so le 50%" prompt="Co = 1/2 số thanh chờ L, 1/2 chờ 2L + KC mối nối" type="list">
       <formula1>LIST!$W$2:$W$3</formula1>
@@ -25506,6 +25506,11 @@
           <t>1/T/B</t>
         </is>
       </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -25533,6 +25538,11 @@
           <t>8u8a50</t>
         </is>
       </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -25553,6 +25563,11 @@
       <c r="D8" t="inlineStr">
         <is>
           <t>TL</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>100/300</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
QS_DAM: ghi ten dam cho noi cho thep cho thang / coupler
- Them truong ten dam cho noi cho moi dau dam (Excel V2: S8 / T8 ; V1: dong CHO_TEN ;
  chuoi cho KIEU|LOP|THEP|L|SOLE|TEN).
- MC doc: ghi 'COUPLER / THEP CHO NOI DAM <ten>' canh dim doan cho, ten dam trong vung
  net khuat zone sau ; dai shop: 'MACH NGUNG - COUPLER NOI DAM <ten>'.
- Sua ma unicode chu MACH NGUNG tren dai shop (thieu 1 dau \ trong chuoi LISP).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VnufFRFDfSW7EG6WSRTNkK
</commit_message>
<xml_diff>
--- a/QS_DAM_NhapLieu.xlsx
+++ b/QS_DAM_NhapLieu.xlsx
@@ -788,6 +788,7 @@
       <text>
         <t>THÉP CHỜ 2 ĐẦU DẦM (khi đầu dầm là mạch ngừng, chờ sang zone / đợt đổ sau)
 • Cho thang: thép kéo thẳng ra ngoài đầu dầm đoạn L chờ, không bẻ ke.
+• Tên dầm chờ nối (S8 / T8): ghi 'THÉP CHỜ / COUPLER NỐI DẦM …' trên MC dọc, shop và tên dầm trong vùng nét khuất.
 • Coupler: thép dừng tại mép (L chờ = 0) hoặc kéo ra ngoài mép: 100, hoặc so le 100/300 (½ số thanh 100, ½ số thanh 300).
 • So le: 1/2 số thanh chờ L, 1/2 chờ 2L + KC mối nối.
 Bản vẽ có nét khuất dầm zone sau, đường MẠCH NGỪNG, dim L chờ; QS_SHOPDAM cắt đúng chiều dài.
@@ -964,6 +965,7 @@
       <text>
         <t>THÉP CHỜ 2 ĐẦU DẦM (khi đầu dầm là mạch ngừng, chờ sang zone / đợt đổ sau)
 • Cho thang: thép kéo thẳng ra ngoài đầu dầm đoạn L chờ, không bẻ ke.
+• Tên dầm chờ nối (S8 / T8): ghi 'THÉP CHỜ / COUPLER NỐI DẦM …' trên MC dọc, shop và tên dầm trong vùng nét khuất.
 • Coupler: thép dừng tại mép (L chờ = 0) hoặc kéo ra ngoài mép: 100, hoặc so le 100/300 (½ số thanh 100, ½ số thanh 300).
 • So le: 1/2 số thanh chờ L, 1/2 chờ 2L + KC mối nối.
 Bản vẽ có nét khuất dầm zone sau, đường MẠCH NGỪNG, dim L chờ; QS_SHOPDAM cắt đúng chiều dài.
@@ -1428,7 +1430,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>• THÉP CHỜ 2 ĐẦU DẦM (S3:T7): kiểu (Khong / Cho thang / Coupler), lớp (TBG, TB, T, B), thanh (Tat ca / Chay suot), L chờ (AUTO / 40d / 1200; coupler 0 / 100 / 100/300 so le), so le.
+          <t>• THÉP CHỜ 2 ĐẦU DẦM (S3:T7): kiểu (Khong / Cho thang / Coupler), lớp (TBG, TB, T, B), thanh (Tat ca / Chay suot), L chờ (AUTO / 40d / 1200; coupler 0 / 100 / 100/300 so le), tên dầm chờ nối (S8:T8), so le.
 • TÙY CHỌN SÀN (Y2:Y3): tai sàn 2 ben / Trai / Phai / Khong, sàn lật – dùng khi F7 chỉ là số (nhập mã DCE 150/1, _150 thì bỏ qua Y2:Y3).
 • Dòng 33-35: tọa độ trục, KC trục-trục tính từ bề rộng gối + Ltt + lệch trục; nhập KC trục mặt bằng (dòng 34) → Ltt suy ra (dòng 35, vàng nếu lệch Ltt đang nhập).
 • Dòng 37-42: kiểm tra As (cm²) bố trí / yêu cầu – thép chạy suốt hiệu dụng (có tính đổi thép dòng 23/25) + tăng cường lớp 1..5; gối tách trái/phải.
@@ -2439,6 +2441,15 @@
       <c r="L8" s="9" t="n"/>
       <c r="M8" s="9" t="n"/>
       <c r="N8" s="10" t="n"/>
+      <c r="P8" s="13" t="inlineStr">
+        <is>
+          <t>Tên dầm chờ nối</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="n"/>
+      <c r="R8" s="6" t="n"/>
+      <c r="S8" s="14" t="inlineStr"/>
+      <c r="T8" s="14" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
@@ -13302,13 +13313,14 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="60">
+  <mergeCells count="61">
     <mergeCell ref="A18:A22"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="C1:N1"/>
     <mergeCell ref="G6:I6"/>
     <mergeCell ref="P2:R2"/>
+    <mergeCell ref="P8:R8"/>
     <mergeCell ref="P1:T1"/>
     <mergeCell ref="G3:I3"/>
     <mergeCell ref="A1:B3"/>
@@ -13471,7 +13483,7 @@
       <formula>LEFT($C$9,1)="✔"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="72">
+  <dataValidations count="73">
     <dataValidation sqref="F2" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Tên dầm" prompt="Tên dầm (ghi trên bản vẽ, tên file CSV)."/>
     <dataValidation sqref="F3" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="b dầm (mm)" prompt="Bề rộng dầm (mm), vd 400."/>
     <dataValidation sqref="F4" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="h dầm (mm)" prompt="Chiều cao dầm (mm), vd 1000."/>
@@ -13530,6 +13542,7 @@
     <dataValidation sqref="S7 T7" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="QS_DAM" error="Chọn giá trị trong danh sách." promptTitle="Chờ so le 50%" prompt="Co = 1/2 số thanh chờ L, 1/2 chờ 2L + KC mối nối" type="list">
       <formula1>LIST!$W$2:$W$3</formula1>
     </dataValidation>
+    <dataValidation sqref="S8 T8" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Tên dầm chờ nối" prompt="Tên dầm / zone sau mà thép chờ (thẳng hoặc coupler) nối sang, vd B138 – ghi lên MC dọc và shop: 'COUPLER NỐI DẦM B138'. Để trống = không ghi."/>
     <dataValidation sqref="Y2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="QS_DAM" error="Chọn giá trị trong danh sách." promptTitle="Tai sàn (phía có sàn)" prompt="2 ben / Trai / Phai / Khong&#10;Chỉ dùng khi F7 là số." type="list">
       <formula1>LIST!$X$2:$X$5</formula1>
     </dataValidation>
@@ -14013,6 +14026,15 @@
       <c r="L8" s="9" t="n"/>
       <c r="M8" s="9" t="n"/>
       <c r="N8" s="10" t="n"/>
+      <c r="P8" s="13" t="inlineStr">
+        <is>
+          <t>Tên dầm chờ nối</t>
+        </is>
+      </c>
+      <c r="Q8" s="6" t="n"/>
+      <c r="R8" s="6" t="n"/>
+      <c r="S8" s="14" t="n"/>
+      <c r="T8" s="14" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
@@ -24548,13 +24570,14 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="60">
+  <mergeCells count="61">
     <mergeCell ref="A18:A22"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="C1:N1"/>
     <mergeCell ref="G6:I6"/>
     <mergeCell ref="P2:R2"/>
+    <mergeCell ref="P8:R8"/>
     <mergeCell ref="P1:T1"/>
     <mergeCell ref="G3:I3"/>
     <mergeCell ref="A1:B3"/>
@@ -24717,7 +24740,7 @@
       <formula>LEFT($C$9,1)="✔"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="72">
+  <dataValidations count="73">
     <dataValidation sqref="F2" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Tên dầm" prompt="Tên dầm (ghi trên bản vẽ, tên file CSV)."/>
     <dataValidation sqref="F3" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="b dầm (mm)" prompt="Bề rộng dầm (mm), vd 400."/>
     <dataValidation sqref="F4" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="h dầm (mm)" prompt="Chiều cao dầm (mm), vd 1000."/>
@@ -24776,6 +24799,7 @@
     <dataValidation sqref="S7 T7" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="QS_DAM" error="Chọn giá trị trong danh sách." promptTitle="Chờ so le 50%" prompt="Co = 1/2 số thanh chờ L, 1/2 chờ 2L + KC mối nối" type="list">
       <formula1>LIST!$W$2:$W$3</formula1>
     </dataValidation>
+    <dataValidation sqref="S8 T8" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Tên dầm chờ nối" prompt="Tên dầm / zone sau mà thép chờ (thẳng hoặc coupler) nối sang, vd B138 – ghi lên MC dọc và shop: 'COUPLER NỐI DẦM B138'. Để trống = không ghi."/>
     <dataValidation sqref="Y2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="QS_DAM" error="Chọn giá trị trong danh sách." promptTitle="Tai sàn (phía có sàn)" prompt="2 ben / Trai / Phai / Khong&#10;Chỉ dùng khi F7 là số." type="list">
       <formula1>LIST!$X$2:$X$5</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
QS_DAM: lenh QS_DAMMB nhan dang dam tren mat bang ket cau -> Excel V2
- Pick diem dau / cuoi tren tim dam: tu do net bien dam (b, can lai tim), cot / vach cat tim
  (goi, L thong thuy), truc cat tim + ten truc (text / block gan dau truc, lech truc so tim goi),
  dam cat ngang (dam phu trong nhip: vi tri tu tim goi + bxh tu text ; dam giao tai cot ;
  goi bien la dam 'bxh'), text ten dam 'B137 (400x1000)' -> ten, b, h.
- Ve tam ket qua (grdraw) + bao cao dong lenh ; copy sheet MAU cua QS_DAM_NhapLieu dang mo
  thanh sheet moi ten dam, ghi F2:F4, dong 11, 24-29 (chuoi co / - duoc giu dang text).
- QS_DAMSET trang 6 (MBKC): mau layer truc / ten truc / cot / dam / text, don vi ban ve,
  ban kinh tim ten truc, b toi da, dai + dai gia cuong ghi san ; tuy chon [Mau] pick layer.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VnufFRFDfSW7EG6WSRTNkK
</commit_message>
<xml_diff>
--- a/QS_DAM_NhapLieu.xlsx
+++ b/QS_DAM_NhapLieu.xlsx
@@ -1378,7 +1378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B43"/>
+  <dimension ref="A1:B44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1465,26 +1465,42 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="31" customHeight="1">
+    <row r="8" ht="71.5" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>LẤY TỪ MẶT BẰNG KC</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Lệnh QS_DAMMB (AutoCAD): mở file này (có sheet MAU) → trên MBKC pick điểm ĐẦU và CUỐI dầm trên tim dầm (ngoài 2 gối biên).
+Lệnh tự nhận dạng: bề rộng b (nét biên dầm), gối (cột / vách cắt tim; đầu dầm gối lên dầm → '400x700'), trục + lệch trục,
+dầm phụ trong nhịp (vị trí từ tim gối, b x h từ text), dầm giao tại cột, tên + b x h dầm từ text 'B137 (400x1000)'
+→ copy sheet MAU thành sheet mới tên dầm và ghi F2:F4, dòng 11, 24–29. Thép chủ, tăng cường… nhập tiếp bằng tay.
+Layer nhận dạng: QS_DAMSET trang 6 hoặc tùy chọn [Mau] của lệnh. Luôn kiểm tra lại số liệu trước khi vẽ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="31" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>KÝ HIỆU THÉP</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>3t28 = 3 thanh Ø28 (t, T, d, f, Ø, %%c đều được). 2t28+1t25 = nhiều loại. '-' = không có.
 Gối: 3t28;5t28 = trái 3t28 / phải 5t28 ; ;2t28 = chỉ bên phải ; 2t25; = chỉ bên trái.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="112" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10" ht="112" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>DÒNG 11 (B11 / lưới)</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>DÒNG 11
 • Ô B11: thép chạy suốt TRÊN, vd 3t28 (2t28+1t25 nếu nhiều loại).
@@ -1497,13 +1513,13 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="71.5" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11" ht="71.5" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>DÒNG 12 (B12 / lưới)</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>DÒNG 12
 • Ô B12: thép chạy suốt DƯỚI, vd 3t28.
@@ -1513,13 +1529,13 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="58" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12" ht="58" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>DÒNG 13-17</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>THÉP TĂNG CƯỜNG LỚP TRÊN (dòng 13 = lớp 1 ... 17 = lớp 5)
 • Cột GỐI: thép mũ gối. 3t28 = 2 bên như nhau; 3t28;5t28 = trái;phải; ;2t28 = chỉ bên phải.
@@ -1528,13 +1544,13 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="44.5" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="13" ht="44.5" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>DÒNG 18-22</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>THÉP TĂNG CƯỜNG LỚP DƯỚI (dòng 22 = lớp 1 ... 18 = lớp 5, giống DCE)
 • Cột NHỊP: thép tăng cường bụng nhịp phía dưới.
@@ -1542,13 +1558,13 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="85" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="14" ht="85" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>DÒNG 23</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>DÒNG 23
 • GỐI: ẩn cột khi vẽ (1 trên · 2 dưới · 3 cả hai).
@@ -1559,13 +1575,13 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="44.5" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="15" ht="44.5" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>DÒNG 24</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>DÒNG 24
 • GỐI: kích thước dầm giao tại cột, vd 400x600.
@@ -1573,13 +1589,13 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="44.5" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16" ht="44.5" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>DÒNG 25</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>DÒNG 25
 • GỐI: độ lệch dầm giao tại cột so với tim cột (mm).
@@ -1587,13 +1603,13 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="44.5" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="17" ht="44.5" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>DÒNG 26</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>DÒNG 26
 • GỐI: tên trục (nhiều dòng thì lấy dòng cuối).
@@ -1601,13 +1617,13 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="71.5" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="18" ht="71.5" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>DÒNG 27</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>DÒNG 27
 • GỐI: độ lệch trục so với tim gối (mm).
@@ -1617,13 +1633,13 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="44.5" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="19" ht="44.5" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>DÒNG 28</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>DÒNG 28
 • GỐI: KT dầm giao nằm trong NHỊP BÊN PHẢI gối (400x600 hoặc 400x600/300x600).
@@ -1631,13 +1647,13 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="58" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="20" ht="58" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>DÒNG 29</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>DÒNG 29
 • GỐI: khoảng cách từ TIM gối tới tim dầm giao trong nhịp phải (2000 hoặc 2000/5000).
@@ -1646,62 +1662,62 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>DÒNG 30</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>DÒNG 30 (chỉ cột NHỊP): thép vai bò tại dầm giao, vd 2t16.</t>
-        </is>
-      </c>
-    </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>DÒNG 30</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>DÒNG 30 (chỉ cột NHỊP): thép vai bò tại dầm giao, vd 2t16.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
           <t>F2 – Tên dầm</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Tên dầm (ghi trên bản vẽ, tên file CSV).</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="31" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
+    <row r="23" ht="31" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>F3 – b dầm (mm)</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>b dầm (mm). Nhịp có b khác: nhập ở dòng 12 cột nhịp.
 Móng băng dạng 300/500/500: chưa hỗ trợ (lấy số đầu).</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>F4 – h dầm (mm)</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Chiều cao dầm (mm), vd 1000.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="44.5" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
+    <row r="25" ht="44.5" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>F5 – Số cấu kiện</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Số cấu kiện giống nhau (nhân số lượng thống kê).
 Thêm /T, /B: đặt mối nối bắt buộc cho thép chạy suốt TRÊN / DƯỚI ở mọi nhịp.
@@ -1709,25 +1725,25 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>F6 – Cao trình dầm (m)</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>Cao độ mặt dầm (m), vd -0.100.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="71.5" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+    <row r="27" ht="71.5" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>F7 – h sàn (mm)</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Chiều dày sàn (mm).
 Chỉ nhập số: phía sàn / sàn lật lấy theo ô Y2, Y3.
@@ -1737,25 +1753,25 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="2" t="inlineStr">
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>F8 – Dầm ngắn L(m) &lt;</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>Nhịp có Ltt nhỏ hơn giá trị này (m): đai rải đều 1 bước.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="139" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+    <row r="29" ht="139" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>J2 – Thép gia cường gối</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>HỆ SỐ THÉP GIA CƯỜNG GỐI (J2)
 Dấu phân cách quyết định cách đo:
@@ -1770,13 +1786,13 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="71.5" customHeight="1">
-      <c r="A29" s="2" t="inlineStr">
+    <row r="30" ht="71.5" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>J3 – Thép gia cường nhịp</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>HỆ SỐ THÉP GIA CƯỜNG NHỊP (J3), cùng quy ước dấu / \ | như J2
 a = thép TC dưới bụng nhịp: L - 2aL
@@ -1786,89 +1802,89 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="31" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+    <row r="31" ht="31" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>J4 – Neo thép trên (d)</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>40 = 40d · 10;12-30d/40d · 10-500mm/12-600mm/...
 Trống = QS_DAMSET</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="31" customHeight="1">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="32" ht="31" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>J5 – Neo thép dưới (d)</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>40 = 40d · 10;12-30d/40d · 10-350mm/12-420mm/...
 Trống = QS_DAMSET</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="31" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
+    <row r="33" ht="31" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>J6 – Neo thép giá (d)</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>40 = 40d · 10;12-30d/40d · 10-350mm/...
 Trống = QS_DAMSET</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="2" t="inlineStr">
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>J7 – Tên trục MCN dầm</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>Tên trục ghi ở mặt cắt ngang (lưu, chưa dùng khi vẽ).</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="31" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
+    <row r="35" ht="31" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>J8 – Lệch trục / Ẩn MC dọc</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>Ltt = thêm dim nhịp thông thủy.
 (100, Y, 100/Y: lưu theo DCE, chưa dùng.)</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="2" t="inlineStr">
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>N2 – ĐK thép C đỡ lớp TC</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>Ø thép C đỡ lớp tăng cường (mm). Trống = Ø đai.</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="71.5" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+    <row r="37" ht="71.5" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>N3 – KC thép C đỡ lớp TC</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>KHOẢNG RẢI THÉP C ĐỠ LỚP TĂNG CƯỜNG (mm)
 &gt; 0 : tự phân biệt lúc cần vẽ (có ≥ 2 lớp)
@@ -1878,86 +1894,86 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>N4 – Đai C nối giữa thép giá</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>None / So le / So le 2 / Toàn bộ</t>
-        </is>
-      </c>
-    </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
+          <t>N4 – Đai C nối giữa thép giá</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>None / So le / So le 2 / Toàn bộ</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
           <t>N5 – ĐK đai C nối 2 thép giá</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Ø đai C nối thép giá (mm). Trống = Ø đai.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="31" customHeight="1">
-      <c r="A39" s="2" t="inlineStr">
+    <row r="40" ht="31" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>N6 – KC đai C nối 2 thép giá</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>400 = móc đai C quay LÊN · 400mm = quay XUỐNG
 Trống = theo bước đai chính.</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>N7 – Giật cao độ dầm</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>Mép trên / Mép dưới / Tùy chỉnh (lưu, chưa dùng khi vẽ).</t>
-        </is>
-      </c>
-    </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
+          <t>N7 – Giật cao độ dầm</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Mép trên / Mép dưới / Tùy chỉnh (lưu, chưa dùng khi vẽ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
           <t>N8 – Dày BT lót dưới dầm</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B42" s="3" t="inlineStr">
         <is>
           <t>100 = BT lót dày 100 · 100/50 = dày 100, mở rộng mỗi bên 50 (mm).</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="31" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>CHƯA HỖ TRỢ</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>Giật cấp mép trên / dưới (dòng 23, 25 số đầu ≠ 0), đổi tiết diện, móng băng (F3/F4/B12 dạng a/b/c), giật sàn T.LINK/-100/-200: QS_DAM cảnh báo và bỏ qua / chỉ đổi thép. Các ô J7, N7, J8 (trừ Ltt) được lưu theo DCE nhưng chưa dùng khi vẽ.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="31" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
+          <t>CHƯA HỖ TRỢ</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Giật cấp mép trên / dưới (dòng 23, 25 số đầu ≠ 0), đổi tiết diện, móng băng (F3/F4/B12 dạng a/b/c), giật sàn T.LINK/-100/-200: QS_DAM cảnh báo và bỏ qua / chỉ đổi thép. Các ô J7, N7, J8 (trừ Ltt) được lưu theo DCE nhưng chưa dùng khi vẽ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="31" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
           <t>GIÁ TRỊ MẶC ĐỊNH</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>Neo, hệ số vùng, móc đai, chiều dài nối để trống = lấy theo QS_DAMSET. Các giá trị mặc định CHƯA XÁC NHẬN – kỹ sư phụ trách kiểm tra theo thuyết minh dự án trước khi phát hành.</t>
         </is>

</xml_diff>

<commit_message>
QS_DAMMB: nhan dang truc theo block truc + pick layer truc / ten truc
- Cai dat MBBLKTRUC (ten block truc, wcmatch, ho tro block dong): ten truc lay tu thuoc tinh,
  text trong dinh nghia block, hoac text roi nam trong bong truc.
- Lenh QS_DAMMB them tuy chon [Truc]: chon block truc -> pick 1 duong truc (layer truc) -> pick
  1 ten truc dang text (layer ten truc, Enter neu dung block). [Mau] = them layer cot, dam, text.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VnufFRFDfSW7EG6WSRTNkK
</commit_message>
<xml_diff>
--- a/QS_DAM_NhapLieu.xlsx
+++ b/QS_DAM_NhapLieu.xlsx
@@ -1465,7 +1465,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="71.5" customHeight="1">
+    <row r="8" ht="125.5" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>LẤY TỪ MẶT BẰNG KC</t>
@@ -1477,7 +1477,9 @@
 Lệnh tự nhận dạng: bề rộng b (nét biên dầm), gối (cột / vách cắt tim; đầu dầm gối lên dầm → '400x700'), trục + lệch trục,
 dầm phụ trong nhịp (vị trí từ tim gối, b x h từ text), dầm giao tại cột, tên + b x h dầm từ text 'B137 (400x1000)'
 → copy sheet MAU thành sheet mới tên dầm và ghi F2:F4, dòng 11, 24–29. Thép chủ, tăng cường… nhập tiếp bằng tay.
-Layer nhận dạng: QS_DAMSET trang 6 hoặc tùy chọn [Mau] của lệnh. Luôn kiểm tra lại số liệu trước khi vẽ.</t>
+Trục: tùy chọn [Truc] của lệnh → chọn BLOCK trục (tên trục = thuộc tính / text trong block / text trong bóng trục) → pick 1 đường trục (layer trục)
+→ pick 1 tên trục dạng text (layer tên trục, Enter nếu đã dùng block). [Mau] = thêm layer cột, dầm, text. Sửa ở QS_DAMSET trang 6.
+Luôn kiểm tra lại số liệu trước khi vẽ.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
QS_DAM: dai con theo so luong thep lop 1 tren
- QS_DAMSET trang 7 (DAI CON): di het dam, khai bao vung goi / nhip, tick 'AUTO tra bang theo
  so luong thep' + bang 2..10 thanh (vd 4 thanh = 2_3, 5 thanh = 3,2_4).
- Excel Y5 / Y6 nhan them dang bang rieng cho dam: 4:2_3;5:3,2_4 ; so thanh thieu trong bang
  rieng -> tra bang QS_DAMSET ; bang ghi AUTO -> tu dong cu.
- So thanh lay tai tung mat cat (vung goi co gia cuong / vung nhip tu ra dai con khac nhau).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VnufFRFDfSW7EG6WSRTNkK
</commit_message>
<xml_diff>
--- a/QS_DAM_NhapLieu.xlsx
+++ b/QS_DAM_NhapLieu.xlsx
@@ -805,7 +805,8 @@
 • 2_4 → đai Q (đai kín) ôm từ thanh 2 đến thanh 4
 • 2-4 → đai U từ thanh 2 đến thanh 4
 • ghép nhiều loại: 3,2_4 (đai C thanh 3 + đai Q thanh 2..4)
-• 0 = không có đai con ; AUTO / trống = tự động (QS_DAMSET trang 2)
+• 0 = không có đai con ; AUTO / trống = tra bảng theo số lượng thép (QS_DAMSET trang 7)
+• theo số lượng thép riêng cho dầm: 4:2_3;5:3,2_4 (4 thanh → Q 2..3 ; 5 thanh → C 3 + Q 2..4)
 Vùng gối có gia cường nên số thanh khác vùng nhịp → Y4 = Khong để khai báo riêng vùng gối (Y5) và vùng nhịp (Y6).
 Chỉ số vượt số thanh thực tế được tự thu về thanh cuối.</t>
       </text>
@@ -994,7 +995,8 @@
 • 2_4 → đai Q (đai kín) ôm từ thanh 2 đến thanh 4
 • 2-4 → đai U từ thanh 2 đến thanh 4
 • ghép nhiều loại: 3,2_4 (đai C thanh 3 + đai Q thanh 2..4)
-• 0 = không có đai con ; AUTO / trống = tự động (QS_DAMSET trang 2)
+• 0 = không có đai con ; AUTO / trống = tra bảng theo số lượng thép (QS_DAMSET trang 7)
+• theo số lượng thép riêng cho dầm: 4:2_3;5:3,2_4 (4 thanh → Q 2..3 ; 5 thanh → C 3 + Q 2..4)
 Vùng gối có gia cường nên số thanh khác vùng nhịp → Y4 = Khong để khai báo riêng vùng gối (Y5) và vùng nhịp (Y6).
 Chỉ số vượt số thanh thực tế được tự thu về thanh cuối.</t>
       </text>
@@ -1510,7 +1512,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="85" customHeight="1">
+    <row r="9" ht="112" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>ĐAI CON (Y4:Y6)</t>
@@ -1520,7 +1522,9 @@
         <is>
           <t>Nhánh đai bên trong theo số thứ tự thanh lớp 1 trên (1..n từ trái sang phải): 2 = đai C tại thanh 2 ; 2_4 = đai Q (kín) ôm thanh 2..4 ;
 2-4 = đai U thanh 2..4 ; ghép 3,2_4 ; 0 = không có ; AUTO / trống = tự động.
-Y4 = Co: Y5 áp dụng cả dầm. Y4 = Khong: Y5 cho vùng gối (vùng đai dày 2 đầu nhịp), Y6 cho vùng nhịp. Trống = QS_DAMSET trang 2.
+Theo số lượng thép (số thanh lớp 1 trên tại mặt cắt): 4:2_3;5:3,2_4 ; số thanh không có trong bảng → bảng QS_DAMSET trang 7.
+AUTO / trống → bảng QS_DAMSET trang 7 (2 … 10 thanh) ; bảng ghi AUTO → tự động cũ (1 nhánh mỗi thanh giữa khi ≥ 4 thanh).
+Y4 = Co: Y5 áp dụng cả dầm. Y4 = Khong: Y5 cho vùng gối (vùng đai dày 2 đầu nhịp), Y6 cho vùng nhịp. Trống = QS_DAMSET trang 7.
 Đường kính / bước đai con = đai trong dòng 27 nếu có, không thì theo đai chính của vùng.</t>
         </is>
       </c>
@@ -13639,11 +13643,11 @@
     <dataValidation sqref="Y4" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="QS_DAM" error="Chọn giá trị trong danh sách." promptTitle="Đai con đi hết dầm" prompt="Co = 1 khai báo (Y5) cho cả dầm.&#10;Khong = vùng gối (vùng đai dày 2 đầu nhịp) dùng Y5, vùng nhịp dùng Y6.&#10;Trống = theo QS_DAMSET trang 2." type="list">
       <formula1>LIST!$W$2:$W$3</formula1>
     </dataValidation>
-    <dataValidation sqref="Y5" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Đai con toàn dầm / vùng gối" prompt="Theo số thứ tự thanh lớp 1 trên (trái → phải):&#10;3 = đai C tại thanh 3&#10;2_4 = đai Q (kín) ôm thanh 2..4&#10;2-4 = đai U thanh 2..4&#10;Ghép: 3,2_4 · 0 = không có · AUTO/trống = tự động" type="list">
-      <formula1>LIST!$X$2:$X$10</formula1>
+    <dataValidation sqref="Y5" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Đai con toàn dầm / vùng gối" prompt="Theo số thứ tự thanh lớp 1 trên (trái → phải): 3 = đai C thanh 3 · 2_4 = đai Q ôm thanh 2..4 · 2-4 = đai U · ghép 3,2_4 · 0 = không có&#10;Theo số lượng thép: 4:2_3;5:3,2_4&#10;AUTO/trống = tra bảng QS_DAMSET trang 7" type="list">
+      <formula1>LIST!$X$2:$X$11</formula1>
     </dataValidation>
-    <dataValidation sqref="Y6" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Đai con vùng nhịp" prompt="Dùng khi Y4 = Khong. Cú pháp như Y5: 2 · 2_4 · 2-4 · 3,2_4 · 0 · AUTO" type="list">
-      <formula1>LIST!$X$2:$X$10</formula1>
+    <dataValidation sqref="Y6" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Đai con vùng nhịp" prompt="Dùng khi Y4 = Khong. Cú pháp như Y5: 2 · 2_4 · 2-4 · 3,2_4 · 4:2_3;5:3,2_4 · 0 · AUTO" type="list">
+      <formula1>LIST!$X$2:$X$11</formula1>
     </dataValidation>
     <dataValidation sqref="C11 E11 G11 I11 K11 M11 O11 Q11 S11 U11 W11 Y11 AA11 AC11 AE11 AG11" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Gối: bề rộng (mm)" prompt="300 = cột 300&#10;0 = console (đầu tự do)&#10;220x500 = gối là DẦM 220x500&#10;1000/220 = cột dưới 1000, cột trên 220&#10;1000/200/-400 = cột trên 200 lệch tim -400"/>
     <dataValidation sqref="D11 F11 H11 J11 L11 N11 P11 R11 T11 V11 X11 Z11 AB11 AD11 AF11" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Nhịp: L thông thủy (mm)" prompt="Khoảng cách 2 mép gối (mm).&#10;Để trống = hết dầm (các nhịp phải liền nhau).&#10;Dòng 34-35: suy Ltt từ khoảng cách trục."/>
@@ -24932,11 +24936,11 @@
     <dataValidation sqref="Y4" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="QS_DAM" error="Chọn giá trị trong danh sách." promptTitle="Đai con đi hết dầm" prompt="Co = 1 khai báo (Y5) cho cả dầm.&#10;Khong = vùng gối (vùng đai dày 2 đầu nhịp) dùng Y5, vùng nhịp dùng Y6.&#10;Trống = theo QS_DAMSET trang 2." type="list">
       <formula1>LIST!$W$2:$W$3</formula1>
     </dataValidation>
-    <dataValidation sqref="Y5" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Đai con toàn dầm / vùng gối" prompt="Theo số thứ tự thanh lớp 1 trên (trái → phải):&#10;3 = đai C tại thanh 3&#10;2_4 = đai Q (kín) ôm thanh 2..4&#10;2-4 = đai U thanh 2..4&#10;Ghép: 3,2_4 · 0 = không có · AUTO/trống = tự động" type="list">
-      <formula1>LIST!$X$2:$X$10</formula1>
+    <dataValidation sqref="Y5" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Đai con toàn dầm / vùng gối" prompt="Theo số thứ tự thanh lớp 1 trên (trái → phải): 3 = đai C thanh 3 · 2_4 = đai Q ôm thanh 2..4 · 2-4 = đai U · ghép 3,2_4 · 0 = không có&#10;Theo số lượng thép: 4:2_3;5:3,2_4&#10;AUTO/trống = tra bảng QS_DAMSET trang 7" type="list">
+      <formula1>LIST!$X$2:$X$11</formula1>
     </dataValidation>
-    <dataValidation sqref="Y6" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Đai con vùng nhịp" prompt="Dùng khi Y4 = Khong. Cú pháp như Y5: 2 · 2_4 · 2-4 · 3,2_4 · 0 · AUTO" type="list">
-      <formula1>LIST!$X$2:$X$10</formula1>
+    <dataValidation sqref="Y6" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Đai con vùng nhịp" prompt="Dùng khi Y4 = Khong. Cú pháp như Y5: 2 · 2_4 · 2-4 · 3,2_4 · 4:2_3;5:3,2_4 · 0 · AUTO" type="list">
+      <formula1>LIST!$X$2:$X$11</formula1>
     </dataValidation>
     <dataValidation sqref="C11 E11 G11 I11 K11 M11 O11 Q11 S11 U11 W11 Y11 AA11 AC11 AE11 AG11" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Gối: bề rộng (mm)" prompt="300 = cột 300&#10;0 = console (đầu tự do)&#10;220x500 = gối là DẦM 220x500&#10;1000/220 = cột dưới 1000, cột trên 220&#10;1000/200/-400 = cột trên 200 lệch tim -400"/>
     <dataValidation sqref="D11 F11 H11 J11 L11 N11 P11 R11 T11 V11 X11 Z11 AB11 AD11 AF11" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Nhịp: L thông thủy (mm)" prompt="Khoảng cách 2 mép gối (mm).&#10;Để trống = hết dầm (các nhịp phải liền nhau).&#10;Dòng 34-35: suy Ltt từ khoảng cách trục."/>
@@ -25833,6 +25837,11 @@
           <t>BR</t>
         </is>
       </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>4:2_3;5:3,2_4</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">

</xml_diff>

<commit_message>
QS_DAM: dai con chi tren Excel (dai C / dai U-Q), shop gia 2 kieu cat, dim shop giong DCE
- Bo trang 7 QS_DAMSET; Excel dong 38 = dai C, dong 39 = dai U / Q theo so thanh
  (so don o dong U/Q = dai C), kiem tra so lieu dong 41..42
- Dai 1 nhanh / dai C doc om ngoai thanh lop 1 tren + lop 1 duoi (truoc bi hut)
- Thep C do lop tang cuong ve thang het be rong dai, KC 2 lop >= phi thanh + phi C do
- Tuy chon TCGOIMAX: thep mu goi 2 ben vuon theo nhip lon hon (dai giu nguyen)
- Shop thep gia: GIACAT = 2 thanh noi so le / 1 thanh
- Shop: net dut 2 mep goi xuyen dai shop + dim chieu dai neo tu mat goi;
  dim chieu dai / chan thanh chi hien chu, sat thanh; shop dai uu tien dim canh duoi / trai,
  chu nam giua duong dim (giong DCE)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VnufFRFDfSW7EG6WSRTNkK
</commit_message>
<xml_diff>
--- a/QS_DAM_NhapLieu.xlsx
+++ b/QS_DAM_NhapLieu.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'VD_L1.B137'!$A:$B</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'VD_L1.B137'!$A$1:$AG$41</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'VD_L1.B137'!$A$1:$AG$42</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'MAU'!$A:$B</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'MAU'!$A$1:$AG$41</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'MAU'!$A$1:$AG$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -923,7 +923,7 @@
 • 2_4 → đai Q (đai kín) ôm từ thanh 2 đến thanh 4
 • 2-4 → đai U từ thanh 2 đến thanh 4
 • ghép nhiều loại: 3,2_4 (đai C thanh 3 + đai Q thanh 2..4)
-• 0 = không có đai con ; AUTO / trống = tra bảng dòng 38 (số thanh ở dòng 37) → bảng QS_DAMSET trang 7
+• 0 = không có đai con ; AUTO / trống = tra bảng: dòng 38 đai C + dòng 39 đai U / Q (số thanh ở dòng 37)
 Vùng gối có gia cường nên số thanh khác vùng nhịp → C33 = Khong để khai báo riêng vùng gối (C34) và vùng nhịp (C35).
 Chỉ số vượt số thanh thực tế được tự thu về thanh cuối. QS_DAMXL ghi lại khối này từ dầm đã vẽ.</t>
       </text>
@@ -1120,7 +1120,7 @@
 • 2_4 → đai Q (đai kín) ôm từ thanh 2 đến thanh 4
 • 2-4 → đai U từ thanh 2 đến thanh 4
 • ghép nhiều loại: 3,2_4 (đai C thanh 3 + đai Q thanh 2..4)
-• 0 = không có đai con ; AUTO / trống = tra bảng dòng 38 (số thanh ở dòng 37) → bảng QS_DAMSET trang 7
+• 0 = không có đai con ; AUTO / trống = tra bảng: dòng 38 đai C + dòng 39 đai U / Q (số thanh ở dòng 37)
 Vùng gối có gia cường nên số thanh khác vùng nhịp → C33 = Khong để khai báo riêng vùng gối (C34) và vùng nhịp (C35).
 Chỉ số vượt số thanh thực tế được tự thu về thanh cuối. QS_DAMXL ghi lại khối này từ dầm đã vẽ.</t>
       </text>
@@ -1443,7 +1443,7 @@
         <is>
           <t>1. Mỗi dầm 1 sheet: chuột phải sheet MAU (hoặc sheet ví dụ) → Move or Copy → Create a copy, đổi tên theo dầm.
 2. Nhập ô trắng. Chọn ô sẽ hiện gợi ý; ô có ▼ có danh sách chọn (vẫn gõ tay được, trừ ô bắt buộc chọn).
-3. Xem dòng 9 (TÌNH TRẠNG SỐ LIỆU) và dòng 41 (KIỂM TRA) – sửa hết ô đỏ.
+3. Xem dòng 9 (TÌNH TRẠNG SỐ LIỆU) và dòng 42 (KIỂM TRA) – sửa hết ô đỏ.
 4. AutoCAD / ZWCAD: để sheet dầm cần vẽ ĐANG MỞ trong Excel → lệnh QS_VEDAM → nguồn Excel → chọn điểm mép TRÊN-TRÁI dầm.
 5. QS_SHOPDAM: cắt thép / shop. QS_DAMSET, QS_DAMNOI: cài đặt móc đai, neo, chiều dài nối.
 6. QS_DAMXL: quét chọn tên dầm (hoặc thép) các dầm ĐÃ VẼ → ghi lại toàn bộ số liệu (kể cả đai con, thép chờ, tên nhịp)
@@ -1477,7 +1477,7 @@
   thanh (Tat ca / Chay suot / TỰ ĐIỀN T:3t28;B:2t25), L chờ / sâu khoan (AUTO / 40 = 40d / 1200 mm; coupler 0 / 100 / 100/300 so le),
   so le, dòng 8 = tên dầm chờ nối hoặc ghi chú khoan cấy.
 • TÙY CHỌN SÀN (Y2:Y3): tai sàn 2 ben / Trai / Phai / Khong, sàn lật – dùng khi F7 chỉ là số (nhập mã DCE 150/1, _150 thì bỏ qua Y2:Y3).
-• Dòng 31: tên dầm theo nhịp (ghi dưới MC dọc). Dòng 32–38: ĐAI CON. Dòng 41 + dòng 9: báo thiếu KT gối, thiếu tên trục,
+• Dòng 31: tên dầm theo nhịp (ghi dưới MC dọc). Dòng 32–39: ĐAI CON. Dòng 42 + dòng 9: báo thiếu KT gối, thiếu tên trục,
   thiếu đai, Ltt sai, nhịp đứt quãng, ký hiệu thép sai (ô thép sai tô đỏ).</t>
         </is>
       </c>
@@ -1543,10 +1543,10 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="85" customHeight="1">
+    <row r="10" ht="139" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>ĐAI CON (dòng 32–38)</t>
+          <t>ĐAI CON (dòng 32–39)</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1554,8 +1554,9 @@
           <t>Nhánh đai bên trong theo số thứ tự thanh lớp 1 trên (1..n từ trái sang phải): 2 = đai C tại thanh 2 ; 2_4 = đai Q (kín) ôm thanh 2..4 ;
 2-4 = đai U thanh 2..4 ; ghép 3,2_4 ; 0 = không có ; AUTO / trống = tra bảng.
 C33 = Co: C34 áp dụng cả dầm. C33 = Khong: C34 cho vùng gối (vùng đai dày 2 đầu nhịp), C35 cho vùng nhịp.
-C36 = Co: tra bảng dòng 38 theo số thanh lớp 1 trên tại mặt cắt (2 … 30 thanh, dòng 37); ô trống → bảng QS_DAMSET trang 7.
-Ô trống ở C33:C36 = theo QS_DAMSET trang 7. Đường kính / bước đai con = đai trong dòng 27 nếu có, không thì theo đai chính.</t>
+C36 = Co / trống: tra bảng theo số thanh lớp 1 trên tại mặt cắt (2 … 30 thanh, dòng 37): dòng 38 = ĐAI C (2,4 ; 2_4 = C tại thanh 2..4),
+dòng 39 = ĐAI U / Q (2_4 = Q, 2-4 = U ; số đơn = đai C). Hai dòng cộng lại. Ô trống / C36 = Khong = đai trong tự động (QS_DAMSET trang 2).
+Đường kính / bước đai con = đai trong dòng 27 nếu có, không thì theo đai chính. (Trang 7 QS_DAMSET đã bỏ – đai con chỉ khai trên Excel.)</t>
         </is>
       </c>
     </row>
@@ -2565,7 +2566,7 @@
       </c>
       <c r="B9" s="20" t="n"/>
       <c r="C9" s="21">
-        <f>IF(SUMPRODUCT((MOD(COLUMN(C63:AG63),2)=0)*C63:AG63)=0,"Chưa có nhịp: nhập bề rộng gối + L thông thủy ở dòng 11",IF(SUMPRODUCT((C41:AG41&lt;&gt;"")*(C41:AG41&lt;&gt;"OK"))+((IFERROR(LEFT(LEFT($B$117,FIND("+",$B$117&amp;"+")-1),FIND("t",LEFT($B$117,FIND("+",$B$117&amp;"+")-1))-1)*MID(LEFT($B$117,FIND("+",$B$117&amp;"+")-1),FIND("t",LEFT($B$117,FIND("+",$B$117&amp;"+")-1))+1,2)^2*PI()/400,0)+IFERROR(LEFT(MID($B$117,FIND("+",$B$117&amp;"+")+1,99),FIND("t",MID($B$117,FIND("+",$B$117&amp;"+")+1,99))-1)*MID(MID($B$117,FIND("+",$B$117&amp;"+")+1,99),FIND("t",MID($B$117,FIND("+",$B$117&amp;"+")+1,99))+1,2)^2*PI()/400,0))=0)+((IFERROR(LEFT(LEFT($B$118,FIND("+",$B$118&amp;"+")-1),FIND("t",LEFT($B$118,FIND("+",$B$118&amp;"+")-1))-1)*MID(LEFT($B$118,FIND("+",$B$118&amp;"+")-1),FIND("t",LEFT($B$118,FIND("+",$B$118&amp;"+")-1))+1,2)^2*PI()/400,0)+IFERROR(LEFT(MID($B$118,FIND("+",$B$118&amp;"+")+1,99),FIND("t",MID($B$118,FIND("+",$B$118&amp;"+")+1,99))-1)*MID(MID($B$118,FIND("+",$B$118&amp;"+")+1,99),FIND("t",MID($B$118,FIND("+",$B$118&amp;"+")+1,99))+1,2)^2*PI()/400,0))=0)=0,"✔  Số liệu hợp lệ – "&amp;SUMPRODUCT((MOD(COLUMN(C63:AG63),2)=0)*C63:AG63)&amp;" nhịp, tổng chiều dài dầm L = "&amp;FIXED(SUMIF(C63:AG63,1,C60:AG60),0)&amp;" mm","✖  Có "&amp;(SUMPRODUCT((C41:AG41&lt;&gt;"")*(C41:AG41&lt;&gt;"OK"))+((IFERROR(LEFT(LEFT($B$117,FIND("+",$B$117&amp;"+")-1),FIND("t",LEFT($B$117,FIND("+",$B$117&amp;"+")-1))-1)*MID(LEFT($B$117,FIND("+",$B$117&amp;"+")-1),FIND("t",LEFT($B$117,FIND("+",$B$117&amp;"+")-1))+1,2)^2*PI()/400,0)+IFERROR(LEFT(MID($B$117,FIND("+",$B$117&amp;"+")+1,99),FIND("t",MID($B$117,FIND("+",$B$117&amp;"+")+1,99))-1)*MID(MID($B$117,FIND("+",$B$117&amp;"+")+1,99),FIND("t",MID($B$117,FIND("+",$B$117&amp;"+")+1,99))+1,2)^2*PI()/400,0))=0)+((IFERROR(LEFT(LEFT($B$118,FIND("+",$B$118&amp;"+")-1),FIND("t",LEFT($B$118,FIND("+",$B$118&amp;"+")-1))-1)*MID(LEFT($B$118,FIND("+",$B$118&amp;"+")-1),FIND("t",LEFT($B$118,FIND("+",$B$118&amp;"+")-1))+1,2)^2*PI()/400,0)+IFERROR(LEFT(MID($B$118,FIND("+",$B$118&amp;"+")+1,99),FIND("t",MID($B$118,FIND("+",$B$118&amp;"+")+1,99))-1)*MID(MID($B$118,FIND("+",$B$118&amp;"+")+1,99),FIND("t",MID($B$118,FIND("+",$B$118&amp;"+")+1,99))+1,2)^2*PI()/400,0))=0))&amp;" lỗi – xem dòng 41 (KIỂM TRA SỐ LIỆU) và ô B11 / B12"))</f>
+        <f>IF(SUMPRODUCT((MOD(COLUMN(C63:AG63),2)=0)*C63:AG63)=0,"Chưa có nhịp: nhập bề rộng gối + L thông thủy ở dòng 11",IF(SUMPRODUCT((C42:AG42&lt;&gt;"")*(C42:AG42&lt;&gt;"OK"))+((IFERROR(LEFT(LEFT($B$117,FIND("+",$B$117&amp;"+")-1),FIND("t",LEFT($B$117,FIND("+",$B$117&amp;"+")-1))-1)*MID(LEFT($B$117,FIND("+",$B$117&amp;"+")-1),FIND("t",LEFT($B$117,FIND("+",$B$117&amp;"+")-1))+1,2)^2*PI()/400,0)+IFERROR(LEFT(MID($B$117,FIND("+",$B$117&amp;"+")+1,99),FIND("t",MID($B$117,FIND("+",$B$117&amp;"+")+1,99))-1)*MID(MID($B$117,FIND("+",$B$117&amp;"+")+1,99),FIND("t",MID($B$117,FIND("+",$B$117&amp;"+")+1,99))+1,2)^2*PI()/400,0))=0)+((IFERROR(LEFT(LEFT($B$118,FIND("+",$B$118&amp;"+")-1),FIND("t",LEFT($B$118,FIND("+",$B$118&amp;"+")-1))-1)*MID(LEFT($B$118,FIND("+",$B$118&amp;"+")-1),FIND("t",LEFT($B$118,FIND("+",$B$118&amp;"+")-1))+1,2)^2*PI()/400,0)+IFERROR(LEFT(MID($B$118,FIND("+",$B$118&amp;"+")+1,99),FIND("t",MID($B$118,FIND("+",$B$118&amp;"+")+1,99))-1)*MID(MID($B$118,FIND("+",$B$118&amp;"+")+1,99),FIND("t",MID($B$118,FIND("+",$B$118&amp;"+")+1,99))+1,2)^2*PI()/400,0))=0)=0,"✔  Số liệu hợp lệ – "&amp;SUMPRODUCT((MOD(COLUMN(C63:AG63),2)=0)*C63:AG63)&amp;" nhịp, tổng chiều dài dầm L = "&amp;FIXED(SUMIF(C63:AG63,1,C60:AG60),0)&amp;" mm","✖  Có "&amp;(SUMPRODUCT((C42:AG42&lt;&gt;"")*(C42:AG42&lt;&gt;"OK"))+((IFERROR(LEFT(LEFT($B$117,FIND("+",$B$117&amp;"+")-1),FIND("t",LEFT($B$117,FIND("+",$B$117&amp;"+")-1))-1)*MID(LEFT($B$117,FIND("+",$B$117&amp;"+")-1),FIND("t",LEFT($B$117,FIND("+",$B$117&amp;"+")-1))+1,2)^2*PI()/400,0)+IFERROR(LEFT(MID($B$117,FIND("+",$B$117&amp;"+")+1,99),FIND("t",MID($B$117,FIND("+",$B$117&amp;"+")+1,99))-1)*MID(MID($B$117,FIND("+",$B$117&amp;"+")+1,99),FIND("t",MID($B$117,FIND("+",$B$117&amp;"+")+1,99))+1,2)^2*PI()/400,0))=0)+((IFERROR(LEFT(LEFT($B$118,FIND("+",$B$118&amp;"+")-1),FIND("t",LEFT($B$118,FIND("+",$B$118&amp;"+")-1))-1)*MID(LEFT($B$118,FIND("+",$B$118&amp;"+")-1),FIND("t",LEFT($B$118,FIND("+",$B$118&amp;"+")-1))+1,2)^2*PI()/400,0)+IFERROR(LEFT(MID($B$118,FIND("+",$B$118&amp;"+")+1,99),FIND("t",MID($B$118,FIND("+",$B$118&amp;"+")+1,99))-1)*MID(MID($B$118,FIND("+",$B$118&amp;"+")+1,99),FIND("t",MID($B$118,FIND("+",$B$118&amp;"+")+1,99))+1,2)^2*PI()/400,0))=0))&amp;" lỗi – xem dòng 42 (KIỂM TRA SỐ LIỆU) và ô B11 / B12"))</f>
         <v/>
       </c>
       <c r="D9" s="22" t="n"/>
@@ -3890,7 +3891,7 @@
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="50" t="inlineStr">
         <is>
-          <t>ĐAI CON – NHÁNH ĐAI BÊN TRONG theo vị trí thanh lớp 1 trên (đánh số 1..n từ trái sang phải) · ô trống = theo QS_DAMSET trang 7</t>
+          <t>ĐAI CON – NHÁNH ĐAI BÊN TRONG theo vị trí thanh lớp 1 trên (đánh số 1..n từ trái sang phải) · trống = đai trong tự động</t>
         </is>
       </c>
       <c r="B32" s="51" t="n"/>
@@ -3937,7 +3938,7 @@
       <c r="D33" s="6" t="n"/>
       <c r="E33" s="54" t="inlineStr">
         <is>
-          <t>Co = khai báo ô C34 áp dụng cả dầm · Khong = C34 cho vùng gối (vùng đai dày 2 đầu nhịp), C35 cho vùng nhịp · trống = QS_DAMSET</t>
+          <t>Co / trống = khai báo ô C34 áp dụng cả dầm · Khong = C34 cho vùng gối (vùng đai dày 2 đầu nhịp), C35 cho vùng nhịp</t>
         </is>
       </c>
       <c r="F33" s="6" t="n"/>
@@ -3980,7 +3981,7 @@
       <c r="D34" s="6" t="n"/>
       <c r="E34" s="54" t="inlineStr">
         <is>
-          <t>3 = đai C (1 nhánh) tại thanh 3 · 2_4 = đai Q (kín) ôm thanh 2..4 · 2-4 = đai U · ghép 3,2_4 · 0 = không có · AUTO / trống = tra bảng dòng 38</t>
+          <t>3 = đai C (1 nhánh) tại thanh 3 · 2_4 = đai Q (kín) ôm thanh 2..4 · 2-4 = đai U · ghép 3,2_4 · 0 = không có · AUTO / trống = tra bảng dòng 38 + 39</t>
         </is>
       </c>
       <c r="F34" s="6" t="n"/>
@@ -4066,7 +4067,7 @@
       <c r="D36" s="6" t="n"/>
       <c r="E36" s="54" t="inlineStr">
         <is>
-          <t>Co = khi C34 / C35 là AUTO / trống: tra bảng dòng 38 theo số thanh lớp 1 trên tại mặt cắt (ô trống → bảng QS_DAMSET trang 7) · Khong = đai trong tự động cũ</t>
+          <t>Co / trống = khi C34 / C35 là AUTO / trống: tra bảng dòng 38 (đai C) + 39 (đai U / Q) theo số thanh lớp 1 trên tại mặt cắt · Khong / ô bảng trống = đai trong tự động</t>
         </is>
       </c>
       <c r="F36" s="6" t="n"/>
@@ -4198,7 +4199,7 @@
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="52" t="inlineStr">
         <is>
-          <t>Nhánh đai con theo số thanh</t>
+          <t>Đai C (1 nhánh) theo số thanh</t>
         </is>
       </c>
       <c r="B38" s="6" t="n"/>
@@ -4234,173 +4235,212 @@
       <c r="AF38" s="57" t="inlineStr"/>
       <c r="AG38" s="57" t="inlineStr"/>
     </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="50" t="inlineStr">
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="52" t="inlineStr">
+        <is>
+          <t>Đai U / Q theo số thanh</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="n"/>
+      <c r="C39" s="58" t="n"/>
+      <c r="D39" s="58" t="n"/>
+      <c r="E39" s="58" t="n"/>
+      <c r="F39" s="58" t="n"/>
+      <c r="G39" s="58" t="n"/>
+      <c r="H39" s="58" t="n"/>
+      <c r="I39" s="58" t="n"/>
+      <c r="J39" s="58" t="n"/>
+      <c r="K39" s="58" t="n"/>
+      <c r="L39" s="58" t="n"/>
+      <c r="M39" s="58" t="n"/>
+      <c r="N39" s="58" t="n"/>
+      <c r="O39" s="58" t="n"/>
+      <c r="P39" s="58" t="n"/>
+      <c r="Q39" s="58" t="n"/>
+      <c r="R39" s="58" t="n"/>
+      <c r="S39" s="58" t="n"/>
+      <c r="T39" s="58" t="n"/>
+      <c r="U39" s="58" t="n"/>
+      <c r="V39" s="58" t="n"/>
+      <c r="W39" s="58" t="n"/>
+      <c r="X39" s="58" t="n"/>
+      <c r="Y39" s="58" t="n"/>
+      <c r="Z39" s="58" t="n"/>
+      <c r="AA39" s="58" t="n"/>
+      <c r="AB39" s="58" t="n"/>
+      <c r="AC39" s="58" t="n"/>
+      <c r="AD39" s="58" t="n"/>
+      <c r="AE39" s="58" t="n"/>
+      <c r="AF39" s="57" t="inlineStr"/>
+      <c r="AG39" s="57" t="inlineStr"/>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="50" t="inlineStr">
         <is>
           <t>KIỂM TRA SỐ LIỆU</t>
         </is>
       </c>
-      <c r="B40" s="51" t="n"/>
-      <c r="C40" s="51" t="n"/>
-      <c r="D40" s="51" t="n"/>
-      <c r="E40" s="51" t="n"/>
-      <c r="F40" s="51" t="n"/>
-      <c r="G40" s="51" t="n"/>
-      <c r="H40" s="51" t="n"/>
-      <c r="I40" s="51" t="n"/>
-      <c r="J40" s="51" t="n"/>
-      <c r="K40" s="51" t="n"/>
-      <c r="L40" s="51" t="n"/>
-      <c r="M40" s="51" t="n"/>
-      <c r="N40" s="51" t="n"/>
-      <c r="O40" s="51" t="n"/>
-      <c r="P40" s="51" t="n"/>
-      <c r="Q40" s="51" t="n"/>
-      <c r="R40" s="51" t="n"/>
-      <c r="S40" s="51" t="n"/>
-      <c r="T40" s="51" t="n"/>
-      <c r="U40" s="51" t="n"/>
-      <c r="V40" s="51" t="n"/>
-      <c r="W40" s="51" t="n"/>
-      <c r="X40" s="51" t="n"/>
-      <c r="Y40" s="51" t="n"/>
-      <c r="Z40" s="51" t="n"/>
-      <c r="AA40" s="51" t="n"/>
-      <c r="AB40" s="51" t="n"/>
-      <c r="AC40" s="51" t="n"/>
-      <c r="AD40" s="51" t="n"/>
-      <c r="AE40" s="51" t="n"/>
-      <c r="AF40" s="51" t="n"/>
-      <c r="AG40" s="51" t="n"/>
-    </row>
-    <row r="41" ht="27" customHeight="1">
-      <c r="A41" s="59" t="inlineStr">
+      <c r="B41" s="51" t="n"/>
+      <c r="C41" s="51" t="n"/>
+      <c r="D41" s="51" t="n"/>
+      <c r="E41" s="51" t="n"/>
+      <c r="F41" s="51" t="n"/>
+      <c r="G41" s="51" t="n"/>
+      <c r="H41" s="51" t="n"/>
+      <c r="I41" s="51" t="n"/>
+      <c r="J41" s="51" t="n"/>
+      <c r="K41" s="51" t="n"/>
+      <c r="L41" s="51" t="n"/>
+      <c r="M41" s="51" t="n"/>
+      <c r="N41" s="51" t="n"/>
+      <c r="O41" s="51" t="n"/>
+      <c r="P41" s="51" t="n"/>
+      <c r="Q41" s="51" t="n"/>
+      <c r="R41" s="51" t="n"/>
+      <c r="S41" s="51" t="n"/>
+      <c r="T41" s="51" t="n"/>
+      <c r="U41" s="51" t="n"/>
+      <c r="V41" s="51" t="n"/>
+      <c r="W41" s="51" t="n"/>
+      <c r="X41" s="51" t="n"/>
+      <c r="Y41" s="51" t="n"/>
+      <c r="Z41" s="51" t="n"/>
+      <c r="AA41" s="51" t="n"/>
+      <c r="AB41" s="51" t="n"/>
+      <c r="AC41" s="51" t="n"/>
+      <c r="AD41" s="51" t="n"/>
+      <c r="AE41" s="51" t="n"/>
+      <c r="AF41" s="51" t="n"/>
+      <c r="AG41" s="51" t="n"/>
+    </row>
+    <row r="42" ht="27" customHeight="1">
+      <c r="A42" s="59" t="inlineStr">
         <is>
           <t>Kết quả kiểm tra từng cột</t>
         </is>
       </c>
-      <c r="B41" s="6" t="n"/>
-      <c r="C41" s="60">
+      <c r="B42" s="6" t="n"/>
+      <c r="C42" s="60">
         <f>IF(C63=0,"",IF(C60="","Thiếu KT gối",IF(C26="","Thiếu tên trục",IF(C116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="D41" s="60">
+      <c r="D42" s="60">
         <f>IF(D63=0,IF(D11="","","Sai Ltt"),IF(FALSE,"Nhịp đứt quãng",IF(D26="","Thiếu đai",IF(D116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="E41" s="60">
+      <c r="E42" s="60">
         <f>IF(E63=0,"",IF(E60="","Thiếu KT gối",IF(E26="","Thiếu tên trục",IF(E116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="F41" s="60">
+      <c r="F42" s="60">
         <f>IF(F63=0,IF(F11="","","Sai Ltt"),IF(AND(D$63=0,F63=1),"Nhịp đứt quãng",IF(F26="","Thiếu đai",IF(F116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="G41" s="60">
+      <c r="G42" s="60">
         <f>IF(G63=0,"",IF(G60="","Thiếu KT gối",IF(G26="","Thiếu tên trục",IF(G116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="H41" s="60">
+      <c r="H42" s="60">
         <f>IF(H63=0,IF(H11="","","Sai Ltt"),IF(AND(F$63=0,H63=1),"Nhịp đứt quãng",IF(H26="","Thiếu đai",IF(H116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="I41" s="60">
+      <c r="I42" s="60">
         <f>IF(I63=0,"",IF(I60="","Thiếu KT gối",IF(I26="","Thiếu tên trục",IF(I116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="J41" s="60">
+      <c r="J42" s="60">
         <f>IF(J63=0,IF(J11="","","Sai Ltt"),IF(AND(H$63=0,J63=1),"Nhịp đứt quãng",IF(J26="","Thiếu đai",IF(J116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="K41" s="60">
+      <c r="K42" s="60">
         <f>IF(K63=0,"",IF(K60="","Thiếu KT gối",IF(K26="","Thiếu tên trục",IF(K116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="L41" s="60">
+      <c r="L42" s="60">
         <f>IF(L63=0,IF(L11="","","Sai Ltt"),IF(AND(J$63=0,L63=1),"Nhịp đứt quãng",IF(L26="","Thiếu đai",IF(L116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="M41" s="60">
+      <c r="M42" s="60">
         <f>IF(M63=0,"",IF(M60="","Thiếu KT gối",IF(M26="","Thiếu tên trục",IF(M116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="N41" s="60">
+      <c r="N42" s="60">
         <f>IF(N63=0,IF(N11="","","Sai Ltt"),IF(AND(L$63=0,N63=1),"Nhịp đứt quãng",IF(N26="","Thiếu đai",IF(N116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="O41" s="60">
+      <c r="O42" s="60">
         <f>IF(O63=0,"",IF(O60="","Thiếu KT gối",IF(O26="","Thiếu tên trục",IF(O116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="P41" s="60">
+      <c r="P42" s="60">
         <f>IF(P63=0,IF(P11="","","Sai Ltt"),IF(AND(N$63=0,P63=1),"Nhịp đứt quãng",IF(P26="","Thiếu đai",IF(P116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="Q41" s="60">
+      <c r="Q42" s="60">
         <f>IF(Q63=0,"",IF(Q60="","Thiếu KT gối",IF(Q26="","Thiếu tên trục",IF(Q116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="R41" s="60">
+      <c r="R42" s="60">
         <f>IF(R63=0,IF(R11="","","Sai Ltt"),IF(AND(P$63=0,R63=1),"Nhịp đứt quãng",IF(R26="","Thiếu đai",IF(R116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="S41" s="60">
+      <c r="S42" s="60">
         <f>IF(S63=0,"",IF(S60="","Thiếu KT gối",IF(S26="","Thiếu tên trục",IF(S116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="T41" s="60">
+      <c r="T42" s="60">
         <f>IF(T63=0,IF(T11="","","Sai Ltt"),IF(AND(R$63=0,T63=1),"Nhịp đứt quãng",IF(T26="","Thiếu đai",IF(T116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="U41" s="60">
+      <c r="U42" s="60">
         <f>IF(U63=0,"",IF(U60="","Thiếu KT gối",IF(U26="","Thiếu tên trục",IF(U116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="V41" s="60">
+      <c r="V42" s="60">
         <f>IF(V63=0,IF(V11="","","Sai Ltt"),IF(AND(T$63=0,V63=1),"Nhịp đứt quãng",IF(V26="","Thiếu đai",IF(V116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="W41" s="60">
+      <c r="W42" s="60">
         <f>IF(W63=0,"",IF(W60="","Thiếu KT gối",IF(W26="","Thiếu tên trục",IF(W116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="X41" s="60">
+      <c r="X42" s="60">
         <f>IF(X63=0,IF(X11="","","Sai Ltt"),IF(AND(V$63=0,X63=1),"Nhịp đứt quãng",IF(X26="","Thiếu đai",IF(X116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="Y41" s="60">
+      <c r="Y42" s="60">
         <f>IF(Y63=0,"",IF(Y60="","Thiếu KT gối",IF(Y26="","Thiếu tên trục",IF(Y116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="Z41" s="60">
+      <c r="Z42" s="60">
         <f>IF(Z63=0,IF(Z11="","","Sai Ltt"),IF(AND(X$63=0,Z63=1),"Nhịp đứt quãng",IF(Z26="","Thiếu đai",IF(Z116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="AA41" s="60">
+      <c r="AA42" s="60">
         <f>IF(AA63=0,"",IF(AA60="","Thiếu KT gối",IF(AA26="","Thiếu tên trục",IF(AA116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="AB41" s="60">
+      <c r="AB42" s="60">
         <f>IF(AB63=0,IF(AB11="","","Sai Ltt"),IF(AND(Z$63=0,AB63=1),"Nhịp đứt quãng",IF(AB26="","Thiếu đai",IF(AB116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="AC41" s="60">
+      <c r="AC42" s="60">
         <f>IF(AC63=0,"",IF(AC60="","Thiếu KT gối",IF(AC26="","Thiếu tên trục",IF(AC116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="AD41" s="60">
+      <c r="AD42" s="60">
         <f>IF(AD63=0,IF(AD11="","","Sai Ltt"),IF(AND(AB$63=0,AD63=1),"Nhịp đứt quãng",IF(AD26="","Thiếu đai",IF(AD116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="AE41" s="60">
+      <c r="AE42" s="60">
         <f>IF(AE63=0,"",IF(AE60="","Thiếu KT gối",IF(AE26="","Thiếu tên trục",IF(AE116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="AF41" s="60">
+      <c r="AF42" s="60">
         <f>IF(AF63=0,IF(AF11="","","Sai Ltt"),IF(AND(AD$63=0,AF63=1),"Nhịp đứt quãng",IF(AF26="","Thiếu đai",IF(AF116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="AG41" s="60">
+      <c r="AG42" s="60">
         <f>IF(AG63=0,"",IF(AG60="","Thiếu KT gối",IF(AG26="","Thiếu tên trục",IF(AG116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
@@ -11782,7 +11822,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="66">
+  <mergeCells count="67">
     <mergeCell ref="C34:D34"/>
     <mergeCell ref="A18:A22"/>
     <mergeCell ref="A24:B24"/>
@@ -11796,6 +11836,7 @@
     <mergeCell ref="P1:T1"/>
     <mergeCell ref="A36:B36"/>
     <mergeCell ref="G3:I3"/>
+    <mergeCell ref="A41:AG41"/>
     <mergeCell ref="A1:B3"/>
     <mergeCell ref="C35:D35"/>
     <mergeCell ref="C2:E2"/>
@@ -11805,7 +11846,6 @@
     <mergeCell ref="K2:M2"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="G5:I5"/>
-    <mergeCell ref="A41:B41"/>
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="A37:B37"/>
     <mergeCell ref="G4:I4"/>
@@ -11822,6 +11862,7 @@
     <mergeCell ref="K6:M6"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="E34:AG34"/>
+    <mergeCell ref="A42:B42"/>
     <mergeCell ref="C36:D36"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="V3:X3"/>
@@ -11837,7 +11878,6 @@
     <mergeCell ref="G2:I2"/>
     <mergeCell ref="E36:AG36"/>
     <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A40:AG40"/>
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="C5:E5"/>
     <mergeCell ref="K5:M5"/>
@@ -11848,6 +11888,7 @@
     <mergeCell ref="C9:AG9"/>
     <mergeCell ref="G7:I7"/>
     <mergeCell ref="P6:R6"/>
+    <mergeCell ref="A39:B39"/>
     <mergeCell ref="A34:B34"/>
   </mergeCells>
   <conditionalFormatting sqref="C11:AG31">
@@ -11855,15 +11896,15 @@
       <formula>C$64=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C41:AG41">
+  <conditionalFormatting sqref="C42:AG42">
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>C$63=0</formula>
     </cfRule>
     <cfRule type="expression" priority="15" dxfId="2">
-      <formula>C41="OK"</formula>
+      <formula>C42="OK"</formula>
     </cfRule>
     <cfRule type="expression" priority="16" dxfId="3">
-      <formula>AND(C41&lt;&gt;"",C41&lt;&gt;"OK")</formula>
+      <formula>AND(C42&lt;&gt;"",C42&lt;&gt;"OK")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C13:AG13">
@@ -11934,7 +11975,7 @@
       <formula>LEFT($C$9,1)="✔"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="76">
+  <dataValidations count="77">
     <dataValidation sqref="F2" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Tên dầm" prompt="Tên dầm (ghi trên bản vẽ, tên file CSV)."/>
     <dataValidation sqref="F3" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="b dầm (mm)" prompt="Bề rộng dầm (mm), vd 400."/>
     <dataValidation sqref="F4" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="h dầm (mm)" prompt="Chiều cao dầm (mm), vd 1000."/>
@@ -11995,7 +12036,7 @@
     </dataValidation>
     <dataValidation sqref="S8 T8" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Tên dầm nối / ghi chú KC" prompt="Chờ / coupler: tên dầm nối sang, vd B138 → 'COUPLER NỐI DẦM B138'.&#10;Khoan cấy: nội dung ghi chú (leader), vd KHOAN CẤY {BAR} SÂU {L} KEO HILTI RE500 · {BAR} {N} {D} {L} tự thay · trống = QS_DAMSET."/>
     <dataValidation sqref="Y2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="QS_DAM" error="Chọn giá trị trong danh sách." promptTitle="Tai sàn (phía có sàn)" prompt="2 ben / Trai / Phai / Khong&#10;Chỉ dùng khi F7 là số." type="list">
-      <formula1>LIST!$Y$2:$Y$5</formula1>
+      <formula1>LIST!$Z$2:$Z$5</formula1>
     </dataValidation>
     <dataValidation sqref="Y3" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="QS_DAM" error="Chọn giá trị trong danh sách." promptTitle="Sàn lật (dầm úp)" prompt="Co = sàn nằm ở đáy dầm. Chỉ dùng khi F7 là số." type="list">
       <formula1>LIST!$W$2:$W$3</formula1>
@@ -12104,19 +12145,22 @@
     <dataValidation sqref="B12" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Thép chạy suốt DƯỚI" prompt="Thép chạy suốt DƯỚI, vd 3t28 · 2t28+1t25.&#10;Đổi thép theo nhịp: dòng 25." type="list">
       <formula1>LIST!$A$2:$A$42</formula1>
     </dataValidation>
-    <dataValidation sqref="C33" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="QS_DAM" error="Chọn giá trị trong danh sách." promptTitle="Đai con đi hết dầm" prompt="Co = khai báo ô C34 áp dụng cả dầm · Khong = C34 cho vùng gối (vùng đai dày 2 đầu nhịp), C35 cho vùng nhịp · trống = QS_DAMSET" type="list">
+    <dataValidation sqref="C33" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="QS_DAM" error="Chọn giá trị trong danh sách." promptTitle="Đai con đi hết dầm" prompt="Co / trống = khai báo ô C34 áp dụng cả dầm · Khong = C34 cho vùng gối (vùng đai dày 2 đầu nhịp), C35 cho vùng nhịp" type="list">
       <formula1>LIST!$W$2:$W$3</formula1>
     </dataValidation>
-    <dataValidation sqref="C34" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Đai con toàn dầm / vùng gối" prompt="3 = đai C (1 nhánh) tại thanh 3 · 2_4 = đai Q (kín) ôm thanh 2..4 · 2-4 = đai U · ghép 3,2_4 · 0 = không có · AUTO / trống = tra bảng dòng 38" type="list">
+    <dataValidation sqref="C34" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Đai con toàn dầm / vùng gối" prompt="3 = đai C (1 nhánh) tại thanh 3 · 2_4 = đai Q (kín) ôm thanh 2..4 · 2-4 = đai U · ghép 3,2_4 · 0 = không có · AUTO / trống = tra bảng dòng 38 + 39" type="list">
       <formula1>LIST!$X$2:$X$12</formula1>
     </dataValidation>
     <dataValidation sqref="C35" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Đai con vùng nhịp" prompt="Dùng khi C33 = Khong. Cú pháp như C34." type="list">
       <formula1>LIST!$X$2:$X$12</formula1>
     </dataValidation>
-    <dataValidation sqref="C36" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="QS_DAM" error="Chọn giá trị trong danh sách." promptTitle="Tra bảng theo số lượng thép" prompt="Co = khi C34 / C35 là AUTO / trống: tra bảng dòng 38 theo số thanh lớp 1 trên tại mặt cắt (ô trống → bảng QS_DAMSET trang 7) · Khong = đai trong tự động cũ" type="list">
+    <dataValidation sqref="C36" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="QS_DAM" error="Chọn giá trị trong danh sách." promptTitle="Tra bảng theo số lượng thép" prompt="Co / trống = khi C34 / C35 là AUTO / trống: tra bảng dòng 38 (đai C) + 39 (đai U / Q) theo số thanh lớp 1 trên tại mặt cắt · Khong / ô bảng trống = đai trong tự động" type="list">
       <formula1>LIST!$W$2:$W$3</formula1>
     </dataValidation>
-    <dataValidation sqref="C38 D38 E38 F38 G38 H38 I38 J38 K38 L38 M38 N38 O38 P38 Q38 R38 S38 T38 U38 V38 W38 X38 Y38 Z38 AA38 AB38 AC38 AD38 AE38" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Đai con theo số thanh" prompt="Số thanh lớp 1 trên ở dòng 37.&#10;2 = đai C thanh 2 · 2_3 = đai Q thanh 2..3 · 2-4 = đai U · 3,2_4 · 0 = không · trống = QS_DAMSET trang 7" type="list">
+    <dataValidation sqref="C38 D38 E38 F38 G38 H38 I38 J38 K38 L38 M38 N38 O38 P38 Q38 R38 S38 T38 U38 V38 W38 X38 Y38 Z38 AA38 AB38 AC38 AD38 AE38" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Đai C theo số thanh" prompt="Số thanh lớp 1 trên ở dòng 37.&#10;Đai C (1 nhánh) tại thanh: 2 · 2,4 · 2_4 (= C tại thanh 2, 3, 4) · 0 = không · trống = không có đai C" type="list">
+      <formula1>LIST!$Y$2:$Y$8</formula1>
+    </dataValidation>
+    <dataValidation sqref="C39 D39 E39 F39 G39 H39 I39 J39 K39 L39 M39 N39 O39 P39 Q39 R39 S39 T39 U39 V39 W39 X39 Y39 Z39 AA39 AB39 AC39 AD39 AE39" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Đai U / Q theo số thanh" prompt="2_4 = đai Q (kín) ôm thanh 2..4 · 2-4 = đai U · ghép 2_3,4_5 · số đơn (vd 2) = đai C tại thanh 2 · trống = không có" type="list">
       <formula1>LIST!$X$2:$X$12</formula1>
     </dataValidation>
   </dataValidations>
@@ -12508,7 +12552,7 @@
       </c>
       <c r="B9" s="20" t="n"/>
       <c r="C9" s="21">
-        <f>IF(SUMPRODUCT((MOD(COLUMN(C63:AG63),2)=0)*C63:AG63)=0,"Chưa có nhịp: nhập bề rộng gối + L thông thủy ở dòng 11",IF(SUMPRODUCT((C41:AG41&lt;&gt;"")*(C41:AG41&lt;&gt;"OK"))+((IFERROR(LEFT(LEFT($B$117,FIND("+",$B$117&amp;"+")-1),FIND("t",LEFT($B$117,FIND("+",$B$117&amp;"+")-1))-1)*MID(LEFT($B$117,FIND("+",$B$117&amp;"+")-1),FIND("t",LEFT($B$117,FIND("+",$B$117&amp;"+")-1))+1,2)^2*PI()/400,0)+IFERROR(LEFT(MID($B$117,FIND("+",$B$117&amp;"+")+1,99),FIND("t",MID($B$117,FIND("+",$B$117&amp;"+")+1,99))-1)*MID(MID($B$117,FIND("+",$B$117&amp;"+")+1,99),FIND("t",MID($B$117,FIND("+",$B$117&amp;"+")+1,99))+1,2)^2*PI()/400,0))=0)+((IFERROR(LEFT(LEFT($B$118,FIND("+",$B$118&amp;"+")-1),FIND("t",LEFT($B$118,FIND("+",$B$118&amp;"+")-1))-1)*MID(LEFT($B$118,FIND("+",$B$118&amp;"+")-1),FIND("t",LEFT($B$118,FIND("+",$B$118&amp;"+")-1))+1,2)^2*PI()/400,0)+IFERROR(LEFT(MID($B$118,FIND("+",$B$118&amp;"+")+1,99),FIND("t",MID($B$118,FIND("+",$B$118&amp;"+")+1,99))-1)*MID(MID($B$118,FIND("+",$B$118&amp;"+")+1,99),FIND("t",MID($B$118,FIND("+",$B$118&amp;"+")+1,99))+1,2)^2*PI()/400,0))=0)=0,"✔  Số liệu hợp lệ – "&amp;SUMPRODUCT((MOD(COLUMN(C63:AG63),2)=0)*C63:AG63)&amp;" nhịp, tổng chiều dài dầm L = "&amp;FIXED(SUMIF(C63:AG63,1,C60:AG60),0)&amp;" mm","✖  Có "&amp;(SUMPRODUCT((C41:AG41&lt;&gt;"")*(C41:AG41&lt;&gt;"OK"))+((IFERROR(LEFT(LEFT($B$117,FIND("+",$B$117&amp;"+")-1),FIND("t",LEFT($B$117,FIND("+",$B$117&amp;"+")-1))-1)*MID(LEFT($B$117,FIND("+",$B$117&amp;"+")-1),FIND("t",LEFT($B$117,FIND("+",$B$117&amp;"+")-1))+1,2)^2*PI()/400,0)+IFERROR(LEFT(MID($B$117,FIND("+",$B$117&amp;"+")+1,99),FIND("t",MID($B$117,FIND("+",$B$117&amp;"+")+1,99))-1)*MID(MID($B$117,FIND("+",$B$117&amp;"+")+1,99),FIND("t",MID($B$117,FIND("+",$B$117&amp;"+")+1,99))+1,2)^2*PI()/400,0))=0)+((IFERROR(LEFT(LEFT($B$118,FIND("+",$B$118&amp;"+")-1),FIND("t",LEFT($B$118,FIND("+",$B$118&amp;"+")-1))-1)*MID(LEFT($B$118,FIND("+",$B$118&amp;"+")-1),FIND("t",LEFT($B$118,FIND("+",$B$118&amp;"+")-1))+1,2)^2*PI()/400,0)+IFERROR(LEFT(MID($B$118,FIND("+",$B$118&amp;"+")+1,99),FIND("t",MID($B$118,FIND("+",$B$118&amp;"+")+1,99))-1)*MID(MID($B$118,FIND("+",$B$118&amp;"+")+1,99),FIND("t",MID($B$118,FIND("+",$B$118&amp;"+")+1,99))+1,2)^2*PI()/400,0))=0))&amp;" lỗi – xem dòng 41 (KIỂM TRA SỐ LIỆU) và ô B11 / B12"))</f>
+        <f>IF(SUMPRODUCT((MOD(COLUMN(C63:AG63),2)=0)*C63:AG63)=0,"Chưa có nhịp: nhập bề rộng gối + L thông thủy ở dòng 11",IF(SUMPRODUCT((C42:AG42&lt;&gt;"")*(C42:AG42&lt;&gt;"OK"))+((IFERROR(LEFT(LEFT($B$117,FIND("+",$B$117&amp;"+")-1),FIND("t",LEFT($B$117,FIND("+",$B$117&amp;"+")-1))-1)*MID(LEFT($B$117,FIND("+",$B$117&amp;"+")-1),FIND("t",LEFT($B$117,FIND("+",$B$117&amp;"+")-1))+1,2)^2*PI()/400,0)+IFERROR(LEFT(MID($B$117,FIND("+",$B$117&amp;"+")+1,99),FIND("t",MID($B$117,FIND("+",$B$117&amp;"+")+1,99))-1)*MID(MID($B$117,FIND("+",$B$117&amp;"+")+1,99),FIND("t",MID($B$117,FIND("+",$B$117&amp;"+")+1,99))+1,2)^2*PI()/400,0))=0)+((IFERROR(LEFT(LEFT($B$118,FIND("+",$B$118&amp;"+")-1),FIND("t",LEFT($B$118,FIND("+",$B$118&amp;"+")-1))-1)*MID(LEFT($B$118,FIND("+",$B$118&amp;"+")-1),FIND("t",LEFT($B$118,FIND("+",$B$118&amp;"+")-1))+1,2)^2*PI()/400,0)+IFERROR(LEFT(MID($B$118,FIND("+",$B$118&amp;"+")+1,99),FIND("t",MID($B$118,FIND("+",$B$118&amp;"+")+1,99))-1)*MID(MID($B$118,FIND("+",$B$118&amp;"+")+1,99),FIND("t",MID($B$118,FIND("+",$B$118&amp;"+")+1,99))+1,2)^2*PI()/400,0))=0)=0,"✔  Số liệu hợp lệ – "&amp;SUMPRODUCT((MOD(COLUMN(C63:AG63),2)=0)*C63:AG63)&amp;" nhịp, tổng chiều dài dầm L = "&amp;FIXED(SUMIF(C63:AG63,1,C60:AG60),0)&amp;" mm","✖  Có "&amp;(SUMPRODUCT((C42:AG42&lt;&gt;"")*(C42:AG42&lt;&gt;"OK"))+((IFERROR(LEFT(LEFT($B$117,FIND("+",$B$117&amp;"+")-1),FIND("t",LEFT($B$117,FIND("+",$B$117&amp;"+")-1))-1)*MID(LEFT($B$117,FIND("+",$B$117&amp;"+")-1),FIND("t",LEFT($B$117,FIND("+",$B$117&amp;"+")-1))+1,2)^2*PI()/400,0)+IFERROR(LEFT(MID($B$117,FIND("+",$B$117&amp;"+")+1,99),FIND("t",MID($B$117,FIND("+",$B$117&amp;"+")+1,99))-1)*MID(MID($B$117,FIND("+",$B$117&amp;"+")+1,99),FIND("t",MID($B$117,FIND("+",$B$117&amp;"+")+1,99))+1,2)^2*PI()/400,0))=0)+((IFERROR(LEFT(LEFT($B$118,FIND("+",$B$118&amp;"+")-1),FIND("t",LEFT($B$118,FIND("+",$B$118&amp;"+")-1))-1)*MID(LEFT($B$118,FIND("+",$B$118&amp;"+")-1),FIND("t",LEFT($B$118,FIND("+",$B$118&amp;"+")-1))+1,2)^2*PI()/400,0)+IFERROR(LEFT(MID($B$118,FIND("+",$B$118&amp;"+")+1,99),FIND("t",MID($B$118,FIND("+",$B$118&amp;"+")+1,99))-1)*MID(MID($B$118,FIND("+",$B$118&amp;"+")+1,99),FIND("t",MID($B$118,FIND("+",$B$118&amp;"+")+1,99))+1,2)^2*PI()/400,0))=0))&amp;" lỗi – xem dòng 42 (KIỂM TRA SỐ LIỆU) và ô B11 / B12"))</f>
         <v/>
       </c>
       <c r="D9" s="22" t="n"/>
@@ -13541,7 +13585,7 @@
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="50" t="inlineStr">
         <is>
-          <t>ĐAI CON – NHÁNH ĐAI BÊN TRONG theo vị trí thanh lớp 1 trên (đánh số 1..n từ trái sang phải) · ô trống = theo QS_DAMSET trang 7</t>
+          <t>ĐAI CON – NHÁNH ĐAI BÊN TRONG theo vị trí thanh lớp 1 trên (đánh số 1..n từ trái sang phải) · trống = đai trong tự động</t>
         </is>
       </c>
       <c r="B32" s="51" t="n"/>
@@ -13588,7 +13632,7 @@
       <c r="D33" s="6" t="n"/>
       <c r="E33" s="54" t="inlineStr">
         <is>
-          <t>Co = khai báo ô C34 áp dụng cả dầm · Khong = C34 cho vùng gối (vùng đai dày 2 đầu nhịp), C35 cho vùng nhịp · trống = QS_DAMSET</t>
+          <t>Co / trống = khai báo ô C34 áp dụng cả dầm · Khong = C34 cho vùng gối (vùng đai dày 2 đầu nhịp), C35 cho vùng nhịp</t>
         </is>
       </c>
       <c r="F33" s="6" t="n"/>
@@ -13631,7 +13675,7 @@
       <c r="D34" s="6" t="n"/>
       <c r="E34" s="54" t="inlineStr">
         <is>
-          <t>3 = đai C (1 nhánh) tại thanh 3 · 2_4 = đai Q (kín) ôm thanh 2..4 · 2-4 = đai U · ghép 3,2_4 · 0 = không có · AUTO / trống = tra bảng dòng 38</t>
+          <t>3 = đai C (1 nhánh) tại thanh 3 · 2_4 = đai Q (kín) ôm thanh 2..4 · 2-4 = đai U · ghép 3,2_4 · 0 = không có · AUTO / trống = tra bảng dòng 38 + 39</t>
         </is>
       </c>
       <c r="F34" s="6" t="n"/>
@@ -13717,7 +13761,7 @@
       <c r="D36" s="6" t="n"/>
       <c r="E36" s="54" t="inlineStr">
         <is>
-          <t>Co = khi C34 / C35 là AUTO / trống: tra bảng dòng 38 theo số thanh lớp 1 trên tại mặt cắt (ô trống → bảng QS_DAMSET trang 7) · Khong = đai trong tự động cũ</t>
+          <t>Co / trống = khi C34 / C35 là AUTO / trống: tra bảng dòng 38 (đai C) + 39 (đai U / Q) theo số thanh lớp 1 trên tại mặt cắt · Khong / ô bảng trống = đai trong tự động</t>
         </is>
       </c>
       <c r="F36" s="6" t="n"/>
@@ -13849,7 +13893,7 @@
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="52" t="inlineStr">
         <is>
-          <t>Nhánh đai con theo số thanh</t>
+          <t>Đai C (1 nhánh) theo số thanh</t>
         </is>
       </c>
       <c r="B38" s="6" t="n"/>
@@ -13885,173 +13929,212 @@
       <c r="AF38" s="57" t="inlineStr"/>
       <c r="AG38" s="57" t="inlineStr"/>
     </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="50" t="inlineStr">
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="52" t="inlineStr">
+        <is>
+          <t>Đai U / Q theo số thanh</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="n"/>
+      <c r="C39" s="58" t="n"/>
+      <c r="D39" s="58" t="n"/>
+      <c r="E39" s="58" t="n"/>
+      <c r="F39" s="58" t="n"/>
+      <c r="G39" s="58" t="n"/>
+      <c r="H39" s="58" t="n"/>
+      <c r="I39" s="58" t="n"/>
+      <c r="J39" s="58" t="n"/>
+      <c r="K39" s="58" t="n"/>
+      <c r="L39" s="58" t="n"/>
+      <c r="M39" s="58" t="n"/>
+      <c r="N39" s="58" t="n"/>
+      <c r="O39" s="58" t="n"/>
+      <c r="P39" s="58" t="n"/>
+      <c r="Q39" s="58" t="n"/>
+      <c r="R39" s="58" t="n"/>
+      <c r="S39" s="58" t="n"/>
+      <c r="T39" s="58" t="n"/>
+      <c r="U39" s="58" t="n"/>
+      <c r="V39" s="58" t="n"/>
+      <c r="W39" s="58" t="n"/>
+      <c r="X39" s="58" t="n"/>
+      <c r="Y39" s="58" t="n"/>
+      <c r="Z39" s="58" t="n"/>
+      <c r="AA39" s="58" t="n"/>
+      <c r="AB39" s="58" t="n"/>
+      <c r="AC39" s="58" t="n"/>
+      <c r="AD39" s="58" t="n"/>
+      <c r="AE39" s="58" t="n"/>
+      <c r="AF39" s="57" t="inlineStr"/>
+      <c r="AG39" s="57" t="inlineStr"/>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="50" t="inlineStr">
         <is>
           <t>KIỂM TRA SỐ LIỆU</t>
         </is>
       </c>
-      <c r="B40" s="51" t="n"/>
-      <c r="C40" s="51" t="n"/>
-      <c r="D40" s="51" t="n"/>
-      <c r="E40" s="51" t="n"/>
-      <c r="F40" s="51" t="n"/>
-      <c r="G40" s="51" t="n"/>
-      <c r="H40" s="51" t="n"/>
-      <c r="I40" s="51" t="n"/>
-      <c r="J40" s="51" t="n"/>
-      <c r="K40" s="51" t="n"/>
-      <c r="L40" s="51" t="n"/>
-      <c r="M40" s="51" t="n"/>
-      <c r="N40" s="51" t="n"/>
-      <c r="O40" s="51" t="n"/>
-      <c r="P40" s="51" t="n"/>
-      <c r="Q40" s="51" t="n"/>
-      <c r="R40" s="51" t="n"/>
-      <c r="S40" s="51" t="n"/>
-      <c r="T40" s="51" t="n"/>
-      <c r="U40" s="51" t="n"/>
-      <c r="V40" s="51" t="n"/>
-      <c r="W40" s="51" t="n"/>
-      <c r="X40" s="51" t="n"/>
-      <c r="Y40" s="51" t="n"/>
-      <c r="Z40" s="51" t="n"/>
-      <c r="AA40" s="51" t="n"/>
-      <c r="AB40" s="51" t="n"/>
-      <c r="AC40" s="51" t="n"/>
-      <c r="AD40" s="51" t="n"/>
-      <c r="AE40" s="51" t="n"/>
-      <c r="AF40" s="51" t="n"/>
-      <c r="AG40" s="51" t="n"/>
-    </row>
-    <row r="41" ht="27" customHeight="1">
-      <c r="A41" s="59" t="inlineStr">
+      <c r="B41" s="51" t="n"/>
+      <c r="C41" s="51" t="n"/>
+      <c r="D41" s="51" t="n"/>
+      <c r="E41" s="51" t="n"/>
+      <c r="F41" s="51" t="n"/>
+      <c r="G41" s="51" t="n"/>
+      <c r="H41" s="51" t="n"/>
+      <c r="I41" s="51" t="n"/>
+      <c r="J41" s="51" t="n"/>
+      <c r="K41" s="51" t="n"/>
+      <c r="L41" s="51" t="n"/>
+      <c r="M41" s="51" t="n"/>
+      <c r="N41" s="51" t="n"/>
+      <c r="O41" s="51" t="n"/>
+      <c r="P41" s="51" t="n"/>
+      <c r="Q41" s="51" t="n"/>
+      <c r="R41" s="51" t="n"/>
+      <c r="S41" s="51" t="n"/>
+      <c r="T41" s="51" t="n"/>
+      <c r="U41" s="51" t="n"/>
+      <c r="V41" s="51" t="n"/>
+      <c r="W41" s="51" t="n"/>
+      <c r="X41" s="51" t="n"/>
+      <c r="Y41" s="51" t="n"/>
+      <c r="Z41" s="51" t="n"/>
+      <c r="AA41" s="51" t="n"/>
+      <c r="AB41" s="51" t="n"/>
+      <c r="AC41" s="51" t="n"/>
+      <c r="AD41" s="51" t="n"/>
+      <c r="AE41" s="51" t="n"/>
+      <c r="AF41" s="51" t="n"/>
+      <c r="AG41" s="51" t="n"/>
+    </row>
+    <row r="42" ht="27" customHeight="1">
+      <c r="A42" s="59" t="inlineStr">
         <is>
           <t>Kết quả kiểm tra từng cột</t>
         </is>
       </c>
-      <c r="B41" s="6" t="n"/>
-      <c r="C41" s="60">
+      <c r="B42" s="6" t="n"/>
+      <c r="C42" s="60">
         <f>IF(C63=0,"",IF(C60="","Thiếu KT gối",IF(C26="","Thiếu tên trục",IF(C116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="D41" s="60">
+      <c r="D42" s="60">
         <f>IF(D63=0,IF(D11="","","Sai Ltt"),IF(FALSE,"Nhịp đứt quãng",IF(D26="","Thiếu đai",IF(D116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="E41" s="60">
+      <c r="E42" s="60">
         <f>IF(E63=0,"",IF(E60="","Thiếu KT gối",IF(E26="","Thiếu tên trục",IF(E116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="F41" s="60">
+      <c r="F42" s="60">
         <f>IF(F63=0,IF(F11="","","Sai Ltt"),IF(AND(D$63=0,F63=1),"Nhịp đứt quãng",IF(F26="","Thiếu đai",IF(F116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="G41" s="60">
+      <c r="G42" s="60">
         <f>IF(G63=0,"",IF(G60="","Thiếu KT gối",IF(G26="","Thiếu tên trục",IF(G116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="H41" s="60">
+      <c r="H42" s="60">
         <f>IF(H63=0,IF(H11="","","Sai Ltt"),IF(AND(F$63=0,H63=1),"Nhịp đứt quãng",IF(H26="","Thiếu đai",IF(H116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="I41" s="60">
+      <c r="I42" s="60">
         <f>IF(I63=0,"",IF(I60="","Thiếu KT gối",IF(I26="","Thiếu tên trục",IF(I116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="J41" s="60">
+      <c r="J42" s="60">
         <f>IF(J63=0,IF(J11="","","Sai Ltt"),IF(AND(H$63=0,J63=1),"Nhịp đứt quãng",IF(J26="","Thiếu đai",IF(J116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="K41" s="60">
+      <c r="K42" s="60">
         <f>IF(K63=0,"",IF(K60="","Thiếu KT gối",IF(K26="","Thiếu tên trục",IF(K116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="L41" s="60">
+      <c r="L42" s="60">
         <f>IF(L63=0,IF(L11="","","Sai Ltt"),IF(AND(J$63=0,L63=1),"Nhịp đứt quãng",IF(L26="","Thiếu đai",IF(L116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="M41" s="60">
+      <c r="M42" s="60">
         <f>IF(M63=0,"",IF(M60="","Thiếu KT gối",IF(M26="","Thiếu tên trục",IF(M116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="N41" s="60">
+      <c r="N42" s="60">
         <f>IF(N63=0,IF(N11="","","Sai Ltt"),IF(AND(L$63=0,N63=1),"Nhịp đứt quãng",IF(N26="","Thiếu đai",IF(N116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="O41" s="60">
+      <c r="O42" s="60">
         <f>IF(O63=0,"",IF(O60="","Thiếu KT gối",IF(O26="","Thiếu tên trục",IF(O116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="P41" s="60">
+      <c r="P42" s="60">
         <f>IF(P63=0,IF(P11="","","Sai Ltt"),IF(AND(N$63=0,P63=1),"Nhịp đứt quãng",IF(P26="","Thiếu đai",IF(P116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="Q41" s="60">
+      <c r="Q42" s="60">
         <f>IF(Q63=0,"",IF(Q60="","Thiếu KT gối",IF(Q26="","Thiếu tên trục",IF(Q116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="R41" s="60">
+      <c r="R42" s="60">
         <f>IF(R63=0,IF(R11="","","Sai Ltt"),IF(AND(P$63=0,R63=1),"Nhịp đứt quãng",IF(R26="","Thiếu đai",IF(R116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="S41" s="60">
+      <c r="S42" s="60">
         <f>IF(S63=0,"",IF(S60="","Thiếu KT gối",IF(S26="","Thiếu tên trục",IF(S116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="T41" s="60">
+      <c r="T42" s="60">
         <f>IF(T63=0,IF(T11="","","Sai Ltt"),IF(AND(R$63=0,T63=1),"Nhịp đứt quãng",IF(T26="","Thiếu đai",IF(T116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="U41" s="60">
+      <c r="U42" s="60">
         <f>IF(U63=0,"",IF(U60="","Thiếu KT gối",IF(U26="","Thiếu tên trục",IF(U116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="V41" s="60">
+      <c r="V42" s="60">
         <f>IF(V63=0,IF(V11="","","Sai Ltt"),IF(AND(T$63=0,V63=1),"Nhịp đứt quãng",IF(V26="","Thiếu đai",IF(V116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="W41" s="60">
+      <c r="W42" s="60">
         <f>IF(W63=0,"",IF(W60="","Thiếu KT gối",IF(W26="","Thiếu tên trục",IF(W116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="X41" s="60">
+      <c r="X42" s="60">
         <f>IF(X63=0,IF(X11="","","Sai Ltt"),IF(AND(V$63=0,X63=1),"Nhịp đứt quãng",IF(X26="","Thiếu đai",IF(X116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="Y41" s="60">
+      <c r="Y42" s="60">
         <f>IF(Y63=0,"",IF(Y60="","Thiếu KT gối",IF(Y26="","Thiếu tên trục",IF(Y116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="Z41" s="60">
+      <c r="Z42" s="60">
         <f>IF(Z63=0,IF(Z11="","","Sai Ltt"),IF(AND(X$63=0,Z63=1),"Nhịp đứt quãng",IF(Z26="","Thiếu đai",IF(Z116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="AA41" s="60">
+      <c r="AA42" s="60">
         <f>IF(AA63=0,"",IF(AA60="","Thiếu KT gối",IF(AA26="","Thiếu tên trục",IF(AA116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="AB41" s="60">
+      <c r="AB42" s="60">
         <f>IF(AB63=0,IF(AB11="","","Sai Ltt"),IF(AND(Z$63=0,AB63=1),"Nhịp đứt quãng",IF(AB26="","Thiếu đai",IF(AB116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="AC41" s="60">
+      <c r="AC42" s="60">
         <f>IF(AC63=0,"",IF(AC60="","Thiếu KT gối",IF(AC26="","Thiếu tên trục",IF(AC116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="AD41" s="60">
+      <c r="AD42" s="60">
         <f>IF(AD63=0,IF(AD11="","","Sai Ltt"),IF(AND(AB$63=0,AD63=1),"Nhịp đứt quãng",IF(AD26="","Thiếu đai",IF(AD116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="AE41" s="60">
+      <c r="AE42" s="60">
         <f>IF(AE63=0,"",IF(AE60="","Thiếu KT gối",IF(AE26="","Thiếu tên trục",IF(AE116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="AF41" s="60">
+      <c r="AF42" s="60">
         <f>IF(AF63=0,IF(AF11="","","Sai Ltt"),IF(AND(AD$63=0,AF63=1),"Nhịp đứt quãng",IF(AF26="","Thiếu đai",IF(AF116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
-      <c r="AG41" s="60">
+      <c r="AG42" s="60">
         <f>IF(AG63=0,"",IF(AG60="","Thiếu KT gối",IF(AG26="","Thiếu tên trục",IF(AG116&gt;0,"Sai KH thép","OK"))))</f>
         <v/>
       </c>
@@ -21433,7 +21516,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="66">
+  <mergeCells count="67">
     <mergeCell ref="C34:D34"/>
     <mergeCell ref="A18:A22"/>
     <mergeCell ref="A24:B24"/>
@@ -21447,6 +21530,7 @@
     <mergeCell ref="P1:T1"/>
     <mergeCell ref="A36:B36"/>
     <mergeCell ref="G3:I3"/>
+    <mergeCell ref="A41:AG41"/>
     <mergeCell ref="A1:B3"/>
     <mergeCell ref="C35:D35"/>
     <mergeCell ref="C2:E2"/>
@@ -21456,7 +21540,6 @@
     <mergeCell ref="K2:M2"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="G5:I5"/>
-    <mergeCell ref="A41:B41"/>
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="A37:B37"/>
     <mergeCell ref="G4:I4"/>
@@ -21473,6 +21556,7 @@
     <mergeCell ref="K6:M6"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="E34:AG34"/>
+    <mergeCell ref="A42:B42"/>
     <mergeCell ref="C36:D36"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="V3:X3"/>
@@ -21488,7 +21572,6 @@
     <mergeCell ref="G2:I2"/>
     <mergeCell ref="E36:AG36"/>
     <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A40:AG40"/>
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="C5:E5"/>
     <mergeCell ref="K5:M5"/>
@@ -21499,6 +21582,7 @@
     <mergeCell ref="C9:AG9"/>
     <mergeCell ref="G7:I7"/>
     <mergeCell ref="P6:R6"/>
+    <mergeCell ref="A39:B39"/>
     <mergeCell ref="A34:B34"/>
   </mergeCells>
   <conditionalFormatting sqref="C11:AG31">
@@ -21506,15 +21590,15 @@
       <formula>C$64=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C41:AG41">
+  <conditionalFormatting sqref="C42:AG42">
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>C$63=0</formula>
     </cfRule>
     <cfRule type="expression" priority="15" dxfId="2">
-      <formula>C41="OK"</formula>
+      <formula>C42="OK"</formula>
     </cfRule>
     <cfRule type="expression" priority="16" dxfId="3">
-      <formula>AND(C41&lt;&gt;"",C41&lt;&gt;"OK")</formula>
+      <formula>AND(C42&lt;&gt;"",C42&lt;&gt;"OK")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C13:AG13">
@@ -21585,7 +21669,7 @@
       <formula>LEFT($C$9,1)="✔"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="76">
+  <dataValidations count="77">
     <dataValidation sqref="F2" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Tên dầm" prompt="Tên dầm (ghi trên bản vẽ, tên file CSV)."/>
     <dataValidation sqref="F3" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="b dầm (mm)" prompt="Bề rộng dầm (mm), vd 400."/>
     <dataValidation sqref="F4" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="h dầm (mm)" prompt="Chiều cao dầm (mm), vd 1000."/>
@@ -21646,7 +21730,7 @@
     </dataValidation>
     <dataValidation sqref="S8 T8" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Tên dầm nối / ghi chú KC" prompt="Chờ / coupler: tên dầm nối sang, vd B138 → 'COUPLER NỐI DẦM B138'.&#10;Khoan cấy: nội dung ghi chú (leader), vd KHOAN CẤY {BAR} SÂU {L} KEO HILTI RE500 · {BAR} {N} {D} {L} tự thay · trống = QS_DAMSET."/>
     <dataValidation sqref="Y2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="QS_DAM" error="Chọn giá trị trong danh sách." promptTitle="Tai sàn (phía có sàn)" prompt="2 ben / Trai / Phai / Khong&#10;Chỉ dùng khi F7 là số." type="list">
-      <formula1>LIST!$Y$2:$Y$5</formula1>
+      <formula1>LIST!$Z$2:$Z$5</formula1>
     </dataValidation>
     <dataValidation sqref="Y3" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="QS_DAM" error="Chọn giá trị trong danh sách." promptTitle="Sàn lật (dầm úp)" prompt="Co = sàn nằm ở đáy dầm. Chỉ dùng khi F7 là số." type="list">
       <formula1>LIST!$W$2:$W$3</formula1>
@@ -21755,19 +21839,22 @@
     <dataValidation sqref="B12" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Thép chạy suốt DƯỚI" prompt="Thép chạy suốt DƯỚI, vd 3t28 · 2t28+1t25.&#10;Đổi thép theo nhịp: dòng 25." type="list">
       <formula1>LIST!$A$2:$A$42</formula1>
     </dataValidation>
-    <dataValidation sqref="C33" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="QS_DAM" error="Chọn giá trị trong danh sách." promptTitle="Đai con đi hết dầm" prompt="Co = khai báo ô C34 áp dụng cả dầm · Khong = C34 cho vùng gối (vùng đai dày 2 đầu nhịp), C35 cho vùng nhịp · trống = QS_DAMSET" type="list">
+    <dataValidation sqref="C33" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="QS_DAM" error="Chọn giá trị trong danh sách." promptTitle="Đai con đi hết dầm" prompt="Co / trống = khai báo ô C34 áp dụng cả dầm · Khong = C34 cho vùng gối (vùng đai dày 2 đầu nhịp), C35 cho vùng nhịp" type="list">
       <formula1>LIST!$W$2:$W$3</formula1>
     </dataValidation>
-    <dataValidation sqref="C34" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Đai con toàn dầm / vùng gối" prompt="3 = đai C (1 nhánh) tại thanh 3 · 2_4 = đai Q (kín) ôm thanh 2..4 · 2-4 = đai U · ghép 3,2_4 · 0 = không có · AUTO / trống = tra bảng dòng 38" type="list">
+    <dataValidation sqref="C34" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Đai con toàn dầm / vùng gối" prompt="3 = đai C (1 nhánh) tại thanh 3 · 2_4 = đai Q (kín) ôm thanh 2..4 · 2-4 = đai U · ghép 3,2_4 · 0 = không có · AUTO / trống = tra bảng dòng 38 + 39" type="list">
       <formula1>LIST!$X$2:$X$12</formula1>
     </dataValidation>
     <dataValidation sqref="C35" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Đai con vùng nhịp" prompt="Dùng khi C33 = Khong. Cú pháp như C34." type="list">
       <formula1>LIST!$X$2:$X$12</formula1>
     </dataValidation>
-    <dataValidation sqref="C36" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="QS_DAM" error="Chọn giá trị trong danh sách." promptTitle="Tra bảng theo số lượng thép" prompt="Co = khi C34 / C35 là AUTO / trống: tra bảng dòng 38 theo số thanh lớp 1 trên tại mặt cắt (ô trống → bảng QS_DAMSET trang 7) · Khong = đai trong tự động cũ" type="list">
+    <dataValidation sqref="C36" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="QS_DAM" error="Chọn giá trị trong danh sách." promptTitle="Tra bảng theo số lượng thép" prompt="Co / trống = khi C34 / C35 là AUTO / trống: tra bảng dòng 38 (đai C) + 39 (đai U / Q) theo số thanh lớp 1 trên tại mặt cắt · Khong / ô bảng trống = đai trong tự động" type="list">
       <formula1>LIST!$W$2:$W$3</formula1>
     </dataValidation>
-    <dataValidation sqref="C38 D38 E38 F38 G38 H38 I38 J38 K38 L38 M38 N38 O38 P38 Q38 R38 S38 T38 U38 V38 W38 X38 Y38 Z38 AA38 AB38 AC38 AD38 AE38" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Đai con theo số thanh" prompt="Số thanh lớp 1 trên ở dòng 37.&#10;2 = đai C thanh 2 · 2_3 = đai Q thanh 2..3 · 2-4 = đai U · 3,2_4 · 0 = không · trống = QS_DAMSET trang 7" type="list">
+    <dataValidation sqref="C38 D38 E38 F38 G38 H38 I38 J38 K38 L38 M38 N38 O38 P38 Q38 R38 S38 T38 U38 V38 W38 X38 Y38 Z38 AA38 AB38 AC38 AD38 AE38" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Đai C theo số thanh" prompt="Số thanh lớp 1 trên ở dòng 37.&#10;Đai C (1 nhánh) tại thanh: 2 · 2,4 · 2_4 (= C tại thanh 2, 3, 4) · 0 = không · trống = không có đai C" type="list">
+      <formula1>LIST!$Y$2:$Y$8</formula1>
+    </dataValidation>
+    <dataValidation sqref="C39 D39 E39 F39 G39 H39 I39 J39 K39 L39 M39 N39 O39 P39 Q39 R39 S39 T39 U39 V39 W39 X39 Y39 Z39 AA39 AB39 AC39 AD39 AE39" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Đai U / Q theo số thanh" prompt="2_4 = đai Q (kín) ôm thanh 2..4 · 2-4 = đai U · ghép 2_3,4_5 · số đơn (vd 2) = đai C tại thanh 2 · trống = không có" type="list">
       <formula1>LIST!$X$2:$X$12</formula1>
     </dataValidation>
   </dataValidations>
@@ -21783,7 +21870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y42"/>
+  <dimension ref="A1:Z42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21811,6 +21898,7 @@
     <col width="14" customWidth="1" min="23" max="23"/>
     <col width="14" customWidth="1" min="24" max="24"/>
     <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -21936,6 +22024,11 @@
       </c>
       <c r="Y1" s="63" t="inlineStr">
         <is>
+          <t>DAICONC</t>
+        </is>
+      </c>
+      <c r="Z1" s="63" t="inlineStr">
+        <is>
           <t>TAISAN</t>
         </is>
       </c>
@@ -22063,6 +22156,11 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
           <t>2 ben</t>
         </is>
       </c>
@@ -22185,6 +22283,11 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
           <t>Trai</t>
         </is>
       </c>
@@ -22297,6 +22400,11 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
+          <t>2,3</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
           <t>Phai</t>
         </is>
       </c>
@@ -22384,6 +22492,11 @@
       </c>
       <c r="Y5" t="inlineStr">
         <is>
+          <t>2,4</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
           <t>Khong</t>
         </is>
       </c>
@@ -22444,6 +22557,11 @@
           <t>2_3</t>
         </is>
       </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>3,4</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -22481,6 +22599,11 @@
           <t>2_4</t>
         </is>
       </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>2,5</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -22511,6 +22634,11 @@
       <c r="X8" t="inlineStr">
         <is>
           <t>2-4</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>

</xml_diff>